<commit_message>
update None to not reported
</commit_message>
<xml_diff>
--- a/advanced-prompting/csv/ground_truth.xlsx
+++ b/advanced-prompting/csv/ground_truth.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kaimingtao/HIVDB/chat_HIVDB_paper/ground truth analysis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kaimingtao/HIVDB/chat_HIVDB_paper/advanced-prompting/csv/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C18B1C1-90DF-F04E-8A26-2B11874F9EE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66595620-9EC5-E748-B3BF-08429EDACFBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="500" windowWidth="37460" windowHeight="20800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="940" yWindow="500" windowWidth="37460" windowHeight="20800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9466" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9466" uniqueCount="312">
   <si>
     <t>PMID</t>
   </si>
@@ -686,9 +686,6 @@
     <t>6078 or 6030</t>
   </si>
   <si>
-    <t>None</t>
-  </si>
-  <si>
     <t>Sanger</t>
   </si>
   <si>
@@ -870,9 +867,6 @@
   </si>
   <si>
     <t>Yes (Only past sequences)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> None</t>
   </si>
   <si>
     <t>249 (uncertain)</t>
@@ -1074,7 +1068,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1095,9 +1089,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1430,7 +1421,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -1513,7 +1504,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>18715920</v>
       </c>
@@ -1833,7 +1824,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>19104010</v>
       </c>
@@ -1950,7 +1941,7 @@
         <v>22</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -2153,7 +2144,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>21115794</v>
       </c>
@@ -2473,7 +2464,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>23749954</v>
       </c>
@@ -2793,7 +2784,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>24227862</v>
       </c>
@@ -3113,7 +3104,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>25637519</v>
       </c>
@@ -3433,7 +3424,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>26246578</v>
       </c>
@@ -3753,7 +3744,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>26311878</v>
       </c>
@@ -4073,7 +4064,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>26559830</v>
       </c>
@@ -4393,7 +4384,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>27124362</v>
       </c>
@@ -4713,7 +4704,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>30803972</v>
       </c>
@@ -5033,7 +5024,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A182">
         <v>31988104</v>
       </c>
@@ -5353,7 +5344,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A198">
         <v>32601157</v>
       </c>
@@ -5673,7 +5664,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A214">
         <v>34516245</v>
       </c>
@@ -5993,7 +5984,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A230">
         <v>35730213</v>
       </c>
@@ -6313,7 +6304,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A246">
         <v>36415058</v>
       </c>
@@ -6633,7 +6624,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A262">
         <v>36519389</v>
       </c>
@@ -6950,10 +6941,10 @@
         <v>7</v>
       </c>
       <c r="F277" s="2" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.2">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="278" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A278">
         <v>36795586</v>
       </c>
@@ -7273,7 +7264,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="294" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A294">
         <v>36920025</v>
       </c>
@@ -7593,7 +7584,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="310" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A310">
         <v>36931676</v>
       </c>
@@ -7830,7 +7821,7 @@
         <v>31</v>
       </c>
       <c r="F321" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="322" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -7913,7 +7904,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="326" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A326">
         <v>36967989</v>
       </c>
@@ -8233,7 +8224,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="342" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A342">
         <v>36982978</v>
       </c>
@@ -8553,7 +8544,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="358" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="358" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A358">
         <v>37052343</v>
       </c>
@@ -8873,7 +8864,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="374" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="374" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A374">
         <v>37071019</v>
       </c>
@@ -8970,7 +8961,7 @@
         <v>22</v>
       </c>
       <c r="F378" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="379" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -9110,7 +9101,7 @@
         <v>31</v>
       </c>
       <c r="F385" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="386" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -9193,7 +9184,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="390" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="390" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A390">
         <v>37358226</v>
       </c>
@@ -9513,7 +9504,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="406" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="406" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A406">
         <v>37540331</v>
       </c>
@@ -9833,7 +9824,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="422" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="422" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A422">
         <v>37541705</v>
       </c>
@@ -10153,7 +10144,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="438" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="438" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A438">
         <v>37632071</v>
       </c>
@@ -10473,7 +10464,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="454" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="454" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A454">
         <v>37649807</v>
       </c>
@@ -10793,7 +10784,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="470" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="470" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A470">
         <v>37662576</v>
       </c>
@@ -11113,7 +11104,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="486" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="486" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A486">
         <v>37716367</v>
       </c>
@@ -11350,7 +11341,7 @@
         <v>31</v>
       </c>
       <c r="F497" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="498" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -11433,7 +11424,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="502" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="502" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A502">
         <v>37872202</v>
       </c>
@@ -11753,7 +11744,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="518" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="518" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A518">
         <v>37910452</v>
       </c>
@@ -12073,7 +12064,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="534" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="534" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A534">
         <v>37966701</v>
       </c>
@@ -12170,7 +12161,7 @@
         <v>22</v>
       </c>
       <c r="F538" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="539" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -12393,7 +12384,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="550" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="550" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A550">
         <v>38005921</v>
       </c>
@@ -12490,7 +12481,7 @@
         <v>22</v>
       </c>
       <c r="F554" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="555" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -12713,7 +12704,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="566" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="566" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A566">
         <v>38022124</v>
       </c>
@@ -13033,7 +13024,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="582" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="582" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A582">
         <v>38031075</v>
       </c>
@@ -13353,7 +13344,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="598" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="598" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A598">
         <v>38033131</v>
       </c>
@@ -13673,7 +13664,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="614" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="614" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A614">
         <v>38140667</v>
       </c>
@@ -13993,7 +13984,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="630" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="630" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A630">
         <v>38142692</v>
       </c>
@@ -14313,7 +14304,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="646" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="646" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A646">
         <v>38427738</v>
       </c>
@@ -14633,7 +14624,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="662" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="662" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A662">
         <v>38864613</v>
       </c>
@@ -14953,7 +14944,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="678" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="678" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A678">
         <v>40938996</v>
       </c>
@@ -15273,7 +15264,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="694" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="694" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A694">
         <v>40965168</v>
       </c>
@@ -15593,7 +15584,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="710" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="710" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A710">
         <v>41091504</v>
       </c>
@@ -15913,7 +15904,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="726" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="726" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A726">
         <v>41093949</v>
       </c>
@@ -16233,7 +16224,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="742" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="742" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A742">
         <v>27009474</v>
       </c>
@@ -16553,7 +16544,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="758" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="758" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A758">
         <v>28559249</v>
       </c>
@@ -16873,7 +16864,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="774" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="774" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A774">
         <v>29373677</v>
       </c>
@@ -17193,7 +17184,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="790" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="790" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A790">
         <v>37147875</v>
       </c>
@@ -17513,7 +17504,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="806" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="806" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A806">
         <v>37554471</v>
       </c>
@@ -17833,7 +17824,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="822" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="822" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A822">
         <v>38072961</v>
       </c>
@@ -18153,7 +18144,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="838" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="838" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A838">
         <v>38152686</v>
       </c>
@@ -18473,7 +18464,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="854" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="854" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A854">
         <v>40431710</v>
       </c>
@@ -18530,7 +18521,7 @@
         <v>18</v>
       </c>
       <c r="F856" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="857" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -18793,7 +18784,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="870" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="870" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A870">
         <v>41088231</v>
       </c>
@@ -18890,7 +18881,7 @@
         <v>22</v>
       </c>
       <c r="F874" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="875" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -19113,7 +19104,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="886" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="886" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A886">
         <v>38058846</v>
       </c>
@@ -19210,7 +19201,7 @@
         <v>22</v>
       </c>
       <c r="F890" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="891" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -19433,7 +19424,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="902" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="902" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A902">
         <v>38090027</v>
       </c>
@@ -19753,7 +19744,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="918" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="918" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A918">
         <v>33855437</v>
       </c>
@@ -20073,7 +20064,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="934" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="934" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A934">
         <v>35945163</v>
       </c>
@@ -20393,7 +20384,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="950" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="950" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A950">
         <v>36597160</v>
       </c>
@@ -20490,7 +20481,7 @@
         <v>22</v>
       </c>
       <c r="F954" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="955" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -20713,7 +20704,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="966" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="966" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A966">
         <v>37957382</v>
       </c>
@@ -21033,7 +21024,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="982" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="982" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A982">
         <v>41056006</v>
       </c>
@@ -21353,7 +21344,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="998" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="998" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A998">
         <v>36659824</v>
       </c>
@@ -21673,7 +21664,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1014" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1014" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1014">
         <v>40713598</v>
       </c>
@@ -21770,7 +21761,7 @@
         <v>22</v>
       </c>
       <c r="F1018" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1019" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -21993,7 +21984,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="1030" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1030" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1030">
         <v>40779404</v>
       </c>
@@ -22090,7 +22081,7 @@
         <v>22</v>
       </c>
       <c r="F1034" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1035" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -22313,7 +22304,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="1046" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1046" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1046">
         <v>41023944</v>
       </c>
@@ -22633,7 +22624,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1062" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1062" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1062">
         <v>40596906</v>
       </c>
@@ -22953,7 +22944,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1078" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1078" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1078">
         <v>37993493</v>
       </c>
@@ -23273,7 +23264,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1094" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1094" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1094">
         <v>38314093</v>
       </c>
@@ -23593,7 +23584,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="1110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1110" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1110">
         <v>40400229</v>
       </c>
@@ -23690,7 +23681,7 @@
         <v>22</v>
       </c>
       <c r="F1114" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1115" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -23913,7 +23904,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1126" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1126">
         <v>37085698</v>
       </c>
@@ -24233,7 +24224,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1142" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1142" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1142">
         <v>30053052</v>
       </c>
@@ -24553,7 +24544,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1158" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1158" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1158">
         <v>35913500</v>
       </c>
@@ -24873,7 +24864,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1174" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1174" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1174">
         <v>37896785</v>
       </c>
@@ -24970,7 +24961,7 @@
         <v>22</v>
       </c>
       <c r="F1178" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1179" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -25193,7 +25184,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1190" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1190" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1190">
         <v>36694270</v>
       </c>
@@ -25290,7 +25281,7 @@
         <v>22</v>
       </c>
       <c r="F1194" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1195" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -25513,7 +25504,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1206" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1206" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1206">
         <v>41130593</v>
       </c>
@@ -25610,7 +25601,7 @@
         <v>22</v>
       </c>
       <c r="F1210" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1211" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -25833,7 +25824,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="1222" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1222" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1222">
         <v>36454248</v>
       </c>
@@ -25930,7 +25921,7 @@
         <v>22</v>
       </c>
       <c r="F1226" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1227" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -26153,7 +26144,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1238" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1238" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1238">
         <v>37914679</v>
       </c>
@@ -26473,7 +26464,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1254" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1254" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1254">
         <v>37537871</v>
       </c>
@@ -26793,7 +26784,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1270" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1270" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1270">
         <v>37039023</v>
       </c>
@@ -27113,7 +27104,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1286" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1286" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1286">
         <v>36851760</v>
       </c>
@@ -27210,7 +27201,7 @@
         <v>22</v>
       </c>
       <c r="F1290" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1291" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -27433,7 +27424,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1302" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1302" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1302">
         <v>37973713</v>
       </c>
@@ -27753,7 +27744,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1318" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1318" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1318">
         <v>37878637</v>
       </c>
@@ -28073,7 +28064,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1334" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1334" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1334">
         <v>37755428</v>
       </c>
@@ -28393,7 +28384,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1350" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1350" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1350">
         <v>40490983</v>
       </c>
@@ -28430,7 +28421,7 @@
         <v>18</v>
       </c>
       <c r="F1351" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="1352" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -28490,7 +28481,7 @@
         <v>22</v>
       </c>
       <c r="F1354" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1355" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -28713,7 +28704,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1366" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1366" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1366">
         <v>36961945</v>
       </c>
@@ -29033,7 +29024,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1382" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1382" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1382">
         <v>41029850</v>
       </c>
@@ -29353,7 +29344,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1398" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1398" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1398">
         <v>36851704</v>
       </c>
@@ -29673,7 +29664,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1414" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1414" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1414">
         <v>40839365</v>
       </c>
@@ -29993,7 +29984,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1430" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1430" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1430">
         <v>40974886</v>
       </c>
@@ -30313,7 +30304,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="1446" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1446" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1446">
         <v>40391923</v>
       </c>
@@ -30633,7 +30624,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1462" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1462" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1462">
         <v>41057785</v>
       </c>
@@ -30649,7 +30640,7 @@
       <c r="E1462" t="s">
         <v>7</v>
       </c>
-      <c r="F1462" s="10">
+      <c r="F1462" s="7">
         <v>235</v>
       </c>
     </row>
@@ -30953,7 +30944,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1478" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1478" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1478">
         <v>41112839</v>
       </c>
@@ -31273,7 +31264,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1494" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1494" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1494">
         <v>37272233</v>
       </c>
@@ -31593,7 +31584,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1510" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1510" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1510">
         <v>38140649</v>
       </c>
@@ -31913,7 +31904,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1526" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1526" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1526">
         <v>37495103</v>
       </c>
@@ -32233,7 +32224,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1542" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1542" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1542">
         <v>40763144</v>
       </c>
@@ -32553,7 +32544,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1558" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1558" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1558">
         <v>38020274</v>
       </c>
@@ -32873,7 +32864,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1574" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1574" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1574">
         <v>41129268</v>
       </c>
@@ -33193,7 +33184,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1590" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1590" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1590">
         <v>37515146</v>
       </c>
@@ -33513,7 +33504,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1606" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1606" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1606">
         <v>37381002</v>
       </c>
@@ -33833,7 +33824,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1622" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1622" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1622">
         <v>40573423</v>
       </c>
@@ -34153,7 +34144,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1638" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1638" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1638">
         <v>36738248</v>
       </c>
@@ -34473,7 +34464,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1654" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1654" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1654">
         <v>37626789</v>
       </c>
@@ -34793,7 +34784,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1670" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1670" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1670">
         <v>37376649</v>
       </c>
@@ -35113,7 +35104,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1686" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1686" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1686">
         <v>37632026</v>
       </c>
@@ -35433,7 +35424,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1702" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1702" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1702">
         <v>37946329</v>
       </c>
@@ -35753,7 +35744,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1718" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1718" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1718">
         <v>40938120</v>
       </c>
@@ -36073,7 +36064,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1734" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1734" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1734">
         <v>37880705</v>
       </c>
@@ -36393,7 +36384,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1750" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1750" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1750">
         <v>37573167</v>
       </c>
@@ -36450,7 +36441,7 @@
         <v>18</v>
       </c>
       <c r="F1752" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="1753" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -36713,7 +36704,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1766" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1766" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1766">
         <v>41004608</v>
       </c>
@@ -37033,7 +37024,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1782" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1782" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1782">
         <v>37029656</v>
       </c>
@@ -37353,7 +37344,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1798" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1798" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1798">
         <v>36779485</v>
       </c>
@@ -37450,7 +37441,7 @@
         <v>22</v>
       </c>
       <c r="F1802" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1803" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -37673,7 +37664,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="1814" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1814" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1814">
         <v>37340869</v>
       </c>
@@ -37770,7 +37761,7 @@
         <v>22</v>
       </c>
       <c r="F1818" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1819" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -37993,7 +37984,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1830" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1830" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1830">
         <v>36751650</v>
       </c>
@@ -38313,7 +38304,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1846" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1846" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1846">
         <v>40431742</v>
       </c>
@@ -38633,7 +38624,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1862" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1862" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1862">
         <v>37546367</v>
       </c>
@@ -38953,7 +38944,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1878" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1878" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1878">
         <v>37976080</v>
       </c>
@@ -39273,7 +39264,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1894" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1894" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1894">
         <v>36571282</v>
       </c>
@@ -39593,7 +39584,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="1910" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1910" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1910">
         <v>38140553</v>
       </c>
@@ -39910,10 +39901,10 @@
         <v>7</v>
       </c>
       <c r="F1925" s="7" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="1926" spans="1:6" x14ac:dyDescent="0.2">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="1926" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1926">
         <v>37976185</v>
       </c>
@@ -39950,7 +39941,7 @@
         <v>18</v>
       </c>
       <c r="F1927" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="1928" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -39970,7 +39961,7 @@
         <v>18</v>
       </c>
       <c r="F1928" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="1929" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40030,7 +40021,7 @@
         <v>22</v>
       </c>
       <c r="F1931" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="1932" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40150,7 +40141,7 @@
         <v>31</v>
       </c>
       <c r="F1937" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="1938" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40213,7 +40204,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="1941" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="1941" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1941">
         <v>40400229</v>
       </c>
@@ -40230,10 +40221,10 @@
         <v>7</v>
       </c>
       <c r="F1941" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="1942" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1942" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1942">
         <v>37112971</v>
       </c>
@@ -40270,7 +40261,7 @@
         <v>18</v>
       </c>
       <c r="F1943" s="7" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="1944" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40330,7 +40321,7 @@
         <v>22</v>
       </c>
       <c r="F1946" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="1947" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40350,7 +40341,7 @@
         <v>22</v>
       </c>
       <c r="F1947" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="1948" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40390,7 +40381,7 @@
         <v>31</v>
       </c>
       <c r="F1949" s="7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="1950" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40533,7 +40524,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="1957" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="1957" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1957">
         <v>40431710</v>
       </c>
@@ -40550,10 +40541,10 @@
         <v>7</v>
       </c>
       <c r="F1957" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="1958" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1958" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1958">
         <v>37585352</v>
       </c>
@@ -40610,7 +40601,7 @@
         <v>18</v>
       </c>
       <c r="F1960" s="7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="1961" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40670,7 +40661,7 @@
         <v>22</v>
       </c>
       <c r="F1963" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="1964" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40790,7 +40781,7 @@
         <v>31</v>
       </c>
       <c r="F1969" s="7" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="1970" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40853,7 +40844,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="1973" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="1973" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1973">
         <v>40431742</v>
       </c>
@@ -40870,10 +40861,10 @@
         <v>7</v>
       </c>
       <c r="F1973" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="1974" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1974" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1974">
         <v>37439411</v>
       </c>
@@ -40910,7 +40901,7 @@
         <v>18</v>
       </c>
       <c r="F1975" s="7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="1976" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40930,7 +40921,7 @@
         <v>18</v>
       </c>
       <c r="F1976" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="1977" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40970,7 +40961,7 @@
         <v>22</v>
       </c>
       <c r="F1978" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="1979" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -40990,7 +40981,7 @@
         <v>22</v>
       </c>
       <c r="F1979" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="1980" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -41073,7 +41064,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="1984" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="1984" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1984">
         <v>40431742</v>
       </c>
@@ -41090,10 +41081,10 @@
         <v>31</v>
       </c>
       <c r="F1984" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="1985" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1985" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1985">
         <v>40431742</v>
       </c>
@@ -41110,7 +41101,7 @@
         <v>31</v>
       </c>
       <c r="F1985" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="1986" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -41173,7 +41164,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="1989" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="1989" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1989">
         <v>40490983</v>
       </c>
@@ -41190,10 +41181,10 @@
         <v>7</v>
       </c>
       <c r="F1989" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="1990" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1990" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1990">
         <v>37279764</v>
       </c>
@@ -41250,7 +41241,7 @@
         <v>18</v>
       </c>
       <c r="F1992" s="7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="1993" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -41290,7 +41281,7 @@
         <v>22</v>
       </c>
       <c r="F1994" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="1995" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -41310,7 +41301,7 @@
         <v>22</v>
       </c>
       <c r="F1995" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="1996" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -41430,7 +41421,7 @@
         <v>31</v>
       </c>
       <c r="F2001" s="7" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2002" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -41493,7 +41484,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2005" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2005" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2005">
         <v>40573423</v>
       </c>
@@ -41510,10 +41501,10 @@
         <v>7</v>
       </c>
       <c r="F2005" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2006" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2006" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2006">
         <v>37593123</v>
       </c>
@@ -41570,7 +41561,7 @@
         <v>18</v>
       </c>
       <c r="F2008" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2009" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -41630,7 +41621,7 @@
         <v>22</v>
       </c>
       <c r="F2011" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2012" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -41713,7 +41704,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2016" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2016" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2016">
         <v>40573423</v>
       </c>
@@ -41730,10 +41721,10 @@
         <v>31</v>
       </c>
       <c r="F2016" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2017" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2017" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2017">
         <v>40573423</v>
       </c>
@@ -41750,7 +41741,7 @@
         <v>31</v>
       </c>
       <c r="F2017" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2018" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -41830,10 +41821,10 @@
         <v>7</v>
       </c>
       <c r="F2021" s="7" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="2022" spans="1:6" x14ac:dyDescent="0.2">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="2022" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2022">
         <v>40872801</v>
       </c>
@@ -41890,7 +41881,7 @@
         <v>18</v>
       </c>
       <c r="F2024" s="7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2025" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -41930,7 +41921,7 @@
         <v>22</v>
       </c>
       <c r="F2026" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2027" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -41950,7 +41941,7 @@
         <v>22</v>
       </c>
       <c r="F2027" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2028" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -42070,7 +42061,7 @@
         <v>31</v>
       </c>
       <c r="F2033" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2034" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -42133,7 +42124,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2037" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2037" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2037">
         <v>40713598</v>
       </c>
@@ -42150,10 +42141,10 @@
         <v>7</v>
       </c>
       <c r="F2037" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2038" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2038" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2038">
         <v>41140464</v>
       </c>
@@ -42210,7 +42201,7 @@
         <v>18</v>
       </c>
       <c r="F2040" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2041" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -42390,7 +42381,7 @@
         <v>31</v>
       </c>
       <c r="F2049" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2050" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -42453,7 +42444,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2053" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2053" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2053">
         <v>40763144</v>
       </c>
@@ -42470,10 +42461,10 @@
         <v>7</v>
       </c>
       <c r="F2053" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2054" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2054" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2054">
         <v>37701387</v>
       </c>
@@ -42490,7 +42481,7 @@
         <v>7</v>
       </c>
       <c r="F2054" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2055" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -42510,7 +42501,7 @@
         <v>18</v>
       </c>
       <c r="F2055" s="7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2056" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -42710,7 +42701,7 @@
         <v>31</v>
       </c>
       <c r="F2065" s="7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2066" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -42773,7 +42764,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2069" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2069" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2069">
         <v>40779404</v>
       </c>
@@ -42790,10 +42781,10 @@
         <v>7</v>
       </c>
       <c r="F2069" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2070" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2070" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2070">
         <v>37941373</v>
       </c>
@@ -42830,7 +42821,7 @@
         <v>18</v>
       </c>
       <c r="F2071" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2072" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -42850,7 +42841,7 @@
         <v>18</v>
       </c>
       <c r="F2072" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2073" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -42890,7 +42881,7 @@
         <v>22</v>
       </c>
       <c r="F2074" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2075" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -42950,7 +42941,7 @@
         <v>31</v>
       </c>
       <c r="F2077" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2078" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43010,7 +43001,7 @@
         <v>31</v>
       </c>
       <c r="F2080" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2081" spans="1:6" ht="30" hidden="1" x14ac:dyDescent="0.2">
@@ -43030,7 +43021,7 @@
         <v>31</v>
       </c>
       <c r="F2081" s="7" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2082" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43093,7 +43084,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2085" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2085" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2085">
         <v>40839365</v>
       </c>
@@ -43110,10 +43101,10 @@
         <v>7</v>
       </c>
       <c r="F2085" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2086" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2086" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2086">
         <v>37674678</v>
       </c>
@@ -43150,7 +43141,7 @@
         <v>18</v>
       </c>
       <c r="F2087" s="7" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2088" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43210,7 +43201,7 @@
         <v>22</v>
       </c>
       <c r="F2090" s="7" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2091" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43230,7 +43221,7 @@
         <v>22</v>
       </c>
       <c r="F2091" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2092" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43310,7 +43301,7 @@
         <v>31</v>
       </c>
       <c r="F2095" s="7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2096" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43350,7 +43341,7 @@
         <v>31</v>
       </c>
       <c r="F2097" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2098" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43413,7 +43404,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2101" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2101">
         <v>40857111</v>
       </c>
@@ -43430,10 +43421,10 @@
         <v>7</v>
       </c>
       <c r="F2101" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2102" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2102" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2102">
         <v>36645792</v>
       </c>
@@ -43470,7 +43461,7 @@
         <v>18</v>
       </c>
       <c r="F2103" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2104" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43490,7 +43481,7 @@
         <v>18</v>
       </c>
       <c r="F2104" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2105" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43530,7 +43521,7 @@
         <v>22</v>
       </c>
       <c r="F2106" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2107" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43550,7 +43541,7 @@
         <v>22</v>
       </c>
       <c r="F2107" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2108" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43670,7 +43661,7 @@
         <v>31</v>
       </c>
       <c r="F2113" s="7" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2114" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43753,7 +43744,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2118" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2118">
         <v>37104815</v>
       </c>
@@ -43810,7 +43801,7 @@
         <v>18</v>
       </c>
       <c r="F2120" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2121" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43850,7 +43841,7 @@
         <v>22</v>
       </c>
       <c r="F2122" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2123" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43870,7 +43861,7 @@
         <v>22</v>
       </c>
       <c r="F2123" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2124" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -43973,7 +43964,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2129" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2129">
         <v>40872801</v>
       </c>
@@ -43990,7 +43981,7 @@
         <v>31</v>
       </c>
       <c r="F2129" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2130" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44070,10 +44061,10 @@
         <v>7</v>
       </c>
       <c r="F2133" s="7" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="2134" spans="1:6" x14ac:dyDescent="0.2">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="2134" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2134">
         <v>37775947</v>
       </c>
@@ -44170,7 +44161,7 @@
         <v>22</v>
       </c>
       <c r="F2138" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2139" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44190,7 +44181,7 @@
         <v>22</v>
       </c>
       <c r="F2139" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2140" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44273,7 +44264,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2144" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2144">
         <v>40938120</v>
       </c>
@@ -44290,10 +44281,10 @@
         <v>31</v>
       </c>
       <c r="F2144" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2145" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2145">
         <v>40938120</v>
       </c>
@@ -44310,7 +44301,7 @@
         <v>31</v>
       </c>
       <c r="F2145" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2146" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44373,7 +44364,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2149" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2149">
         <v>40938996</v>
       </c>
@@ -44390,10 +44381,10 @@
         <v>7</v>
       </c>
       <c r="F2149" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2150" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2150" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2150">
         <v>37327289</v>
       </c>
@@ -44410,7 +44401,7 @@
         <v>7</v>
       </c>
       <c r="F2150" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2151" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44430,7 +44421,7 @@
         <v>18</v>
       </c>
       <c r="F2151" s="7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2152" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44470,7 +44461,7 @@
         <v>22</v>
       </c>
       <c r="F2153" s="7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2154" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44490,7 +44481,7 @@
         <v>22</v>
       </c>
       <c r="F2154" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2155" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44513,7 +44504,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2156" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2156" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2156">
         <v>40938996</v>
       </c>
@@ -44530,7 +44521,7 @@
         <v>22</v>
       </c>
       <c r="F2156" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2157" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44593,7 +44584,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2160" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2160" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2160">
         <v>40938996</v>
       </c>
@@ -44610,10 +44601,10 @@
         <v>31</v>
       </c>
       <c r="F2160" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2161" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2161">
         <v>40938996</v>
       </c>
@@ -44630,7 +44621,7 @@
         <v>31</v>
       </c>
       <c r="F2161" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2162" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44693,7 +44684,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2165" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2165">
         <v>40965168</v>
       </c>
@@ -44710,10 +44701,10 @@
         <v>7</v>
       </c>
       <c r="F2165" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2166" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2166" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2166">
         <v>41012586</v>
       </c>
@@ -44730,7 +44721,7 @@
         <v>7</v>
       </c>
       <c r="F2166" s="7" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="2167" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44750,7 +44741,7 @@
         <v>18</v>
       </c>
       <c r="F2167" s="7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2168" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44810,7 +44801,7 @@
         <v>22</v>
       </c>
       <c r="F2170" s="7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2171" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44830,7 +44821,7 @@
         <v>22</v>
       </c>
       <c r="F2171" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2172" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -44913,7 +44904,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2176" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2176" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2176">
         <v>40965168</v>
       </c>
@@ -44930,10 +44921,10 @@
         <v>31</v>
       </c>
       <c r="F2176" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2177" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2177" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2177">
         <v>40965168</v>
       </c>
@@ -44950,7 +44941,7 @@
         <v>31</v>
       </c>
       <c r="F2177" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2178" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45013,7 +45004,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2181" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2181" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2181">
         <v>40974886</v>
       </c>
@@ -45030,10 +45021,10 @@
         <v>7</v>
       </c>
       <c r="F2181" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2182" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2182" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2182">
         <v>37520425</v>
       </c>
@@ -45070,7 +45061,7 @@
         <v>18</v>
       </c>
       <c r="F2183" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2184" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45090,7 +45081,7 @@
         <v>18</v>
       </c>
       <c r="F2184" s="7" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2185" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45130,7 +45121,7 @@
         <v>22</v>
       </c>
       <c r="F2186" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2187" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45170,7 +45161,7 @@
         <v>22</v>
       </c>
       <c r="F2188" s="7" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2189" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45270,7 +45261,7 @@
         <v>31</v>
       </c>
       <c r="F2193" s="7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2194" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45333,7 +45324,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2197" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2197" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2197">
         <v>41004608</v>
       </c>
@@ -45350,10 +45341,10 @@
         <v>7</v>
       </c>
       <c r="F2197" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2198" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2198" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2198">
         <v>37498738</v>
       </c>
@@ -45390,7 +45381,7 @@
         <v>18</v>
       </c>
       <c r="F2199" s="7" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2200" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45450,7 +45441,7 @@
         <v>22</v>
       </c>
       <c r="F2202" s="7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2203" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45553,7 +45544,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2208" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2208" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2208">
         <v>41004608</v>
       </c>
@@ -45570,10 +45561,10 @@
         <v>31</v>
       </c>
       <c r="F2208" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2209" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2209" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2209">
         <v>41004608</v>
       </c>
@@ -45590,7 +45581,7 @@
         <v>31</v>
       </c>
       <c r="F2209" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2210" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45610,7 +45601,7 @@
         <v>7</v>
       </c>
       <c r="F2210" s="7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2211" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45653,7 +45644,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2213" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2213" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2213">
         <v>41012586</v>
       </c>
@@ -45670,10 +45661,10 @@
         <v>7</v>
       </c>
       <c r="F2213" s="7" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="2214" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2214" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2214">
         <v>37817087</v>
       </c>
@@ -45730,7 +45721,7 @@
         <v>18</v>
       </c>
       <c r="F2216" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2217" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45770,7 +45761,7 @@
         <v>22</v>
       </c>
       <c r="F2218" s="7" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2219" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45790,7 +45781,7 @@
         <v>22</v>
       </c>
       <c r="F2219" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2220" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45810,7 +45801,7 @@
         <v>22</v>
       </c>
       <c r="F2220" s="7" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2221" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45890,7 +45881,7 @@
         <v>31</v>
       </c>
       <c r="F2224" s="7" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2225" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45910,7 +45901,7 @@
         <v>31</v>
       </c>
       <c r="F2225" s="7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2226" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -45973,7 +45964,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2229" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2229" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2229">
         <v>41023944</v>
       </c>
@@ -45990,10 +45981,10 @@
         <v>7</v>
       </c>
       <c r="F2229" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2230" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2230" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2230">
         <v>37920909</v>
       </c>
@@ -46030,7 +46021,7 @@
         <v>18</v>
       </c>
       <c r="F2231" s="7" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2232" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46050,7 +46041,7 @@
         <v>18</v>
       </c>
       <c r="F2232" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2233" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46090,7 +46081,7 @@
         <v>22</v>
       </c>
       <c r="F2234" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2235" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46110,7 +46101,7 @@
         <v>22</v>
       </c>
       <c r="F2235" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2236" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46210,7 +46201,7 @@
         <v>31</v>
       </c>
       <c r="F2240" s="7" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="2241" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46230,7 +46221,7 @@
         <v>31</v>
       </c>
       <c r="F2241" s="7" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="2242" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46290,7 +46281,7 @@
         <v>7</v>
       </c>
       <c r="F2244" s="7" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="2245" spans="1:6" ht="45" hidden="1" x14ac:dyDescent="0.2">
@@ -46310,10 +46301,10 @@
         <v>7</v>
       </c>
       <c r="F2245" s="7" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="2246" spans="1:6" x14ac:dyDescent="0.2">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="2246" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2246">
         <v>37823653</v>
       </c>
@@ -46410,7 +46401,7 @@
         <v>22</v>
       </c>
       <c r="F2250" s="7" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2251" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46430,7 +46421,7 @@
         <v>22</v>
       </c>
       <c r="F2251" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2252" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46530,7 +46521,7 @@
         <v>31</v>
       </c>
       <c r="F2256" s="7" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2257" spans="1:6" ht="30" hidden="1" x14ac:dyDescent="0.2">
@@ -46550,7 +46541,7 @@
         <v>31</v>
       </c>
       <c r="F2257" s="7" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2258" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46613,7 +46604,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2261" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2261" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2261">
         <v>41056006</v>
       </c>
@@ -46630,10 +46621,10 @@
         <v>7</v>
       </c>
       <c r="F2261" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2262" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2262" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2262">
         <v>36706364</v>
       </c>
@@ -46670,7 +46661,7 @@
         <v>18</v>
       </c>
       <c r="F2263" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2264" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46690,7 +46681,7 @@
         <v>18</v>
       </c>
       <c r="F2264" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2265" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46730,7 +46721,7 @@
         <v>22</v>
       </c>
       <c r="F2266" s="7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2267" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46750,7 +46741,7 @@
         <v>22</v>
       </c>
       <c r="F2267" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2268" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46850,7 +46841,7 @@
         <v>31</v>
       </c>
       <c r="F2272" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="2273" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46870,7 +46861,7 @@
         <v>31</v>
       </c>
       <c r="F2273" s="7" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="2274" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46933,7 +46924,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2277" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2277" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2277">
         <v>41057785</v>
       </c>
@@ -46949,11 +46940,11 @@
       <c r="E2277" t="s">
         <v>7</v>
       </c>
-      <c r="F2277" s="8" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2278" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F2277" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2278" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2278">
         <v>40857111</v>
       </c>
@@ -46970,7 +46961,7 @@
         <v>7</v>
       </c>
       <c r="F2278" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="2279" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -46990,7 +46981,7 @@
         <v>18</v>
       </c>
       <c r="F2279" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2280" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47010,7 +47001,7 @@
         <v>18</v>
       </c>
       <c r="F2280" s="8" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="2281" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47050,7 +47041,7 @@
         <v>22</v>
       </c>
       <c r="F2282" s="8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2283" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47070,7 +47061,7 @@
         <v>22</v>
       </c>
       <c r="F2283" s="8" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="2284" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47090,7 +47081,7 @@
         <v>22</v>
       </c>
       <c r="F2284" s="8" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2285" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47170,7 +47161,7 @@
         <v>31</v>
       </c>
       <c r="F2288" s="8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2289" spans="1:6" ht="30" hidden="1" x14ac:dyDescent="0.2">
@@ -47190,7 +47181,7 @@
         <v>31</v>
       </c>
       <c r="F2289" s="8" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="2290" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47270,10 +47261,10 @@
         <v>7</v>
       </c>
       <c r="F2293" s="7" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="2294" spans="1:6" x14ac:dyDescent="0.2">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="2294" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2294">
         <v>37574435</v>
       </c>
@@ -47370,7 +47361,7 @@
         <v>22</v>
       </c>
       <c r="F2298" s="7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2299" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47390,7 +47381,7 @@
         <v>22</v>
       </c>
       <c r="F2299" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2300" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47470,10 +47461,10 @@
         <v>31</v>
       </c>
       <c r="F2303" s="7" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="2304" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="2304" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2304">
         <v>41088231</v>
       </c>
@@ -47490,10 +47481,10 @@
         <v>31</v>
       </c>
       <c r="F2304" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2305" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2305" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2305">
         <v>41088231</v>
       </c>
@@ -47510,7 +47501,7 @@
         <v>31</v>
       </c>
       <c r="F2305" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2306" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47573,7 +47564,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2309" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2309" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2309">
         <v>41091504</v>
       </c>
@@ -47590,10 +47581,10 @@
         <v>7</v>
       </c>
       <c r="F2309" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2310" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2310" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2310">
         <v>37896860</v>
       </c>
@@ -47610,7 +47601,7 @@
         <v>7</v>
       </c>
       <c r="F2310" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2311" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47630,7 +47621,7 @@
         <v>18</v>
       </c>
       <c r="F2311" s="7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2312" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47670,7 +47661,7 @@
         <v>22</v>
       </c>
       <c r="F2313" s="7" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="2314" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47710,10 +47701,10 @@
         <v>22</v>
       </c>
       <c r="F2315" s="7" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="2316" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="2316" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2316">
         <v>41091504</v>
       </c>
@@ -47730,7 +47721,7 @@
         <v>22</v>
       </c>
       <c r="F2316" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2317" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47790,10 +47781,10 @@
         <v>31</v>
       </c>
       <c r="F2319" s="7" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="2320" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="2320" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2320">
         <v>41091504</v>
       </c>
@@ -47810,10 +47801,10 @@
         <v>31</v>
       </c>
       <c r="F2320" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2321" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2321" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2321">
         <v>41091504</v>
       </c>
@@ -47830,7 +47821,7 @@
         <v>31</v>
       </c>
       <c r="F2321" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2322" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47850,7 +47841,7 @@
         <v>7</v>
       </c>
       <c r="F2322" s="7" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2323" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47890,7 +47881,7 @@
         <v>7</v>
       </c>
       <c r="F2324" s="7" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2325" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47910,10 +47901,10 @@
         <v>7</v>
       </c>
       <c r="F2325" s="7" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="2326" spans="1:6" x14ac:dyDescent="0.2">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="2326" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2326">
         <v>36660819</v>
       </c>
@@ -47950,7 +47941,7 @@
         <v>18</v>
       </c>
       <c r="F2327" s="7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2328" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -47970,7 +47961,7 @@
         <v>18</v>
       </c>
       <c r="F2328" s="7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2329" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48030,10 +48021,10 @@
         <v>22</v>
       </c>
       <c r="F2331" s="7" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="2332" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="2332" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2332">
         <v>41093949</v>
       </c>
@@ -48050,7 +48041,7 @@
         <v>22</v>
       </c>
       <c r="F2332" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2333" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48090,7 +48081,7 @@
         <v>31</v>
       </c>
       <c r="F2334" s="7" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2335" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48110,10 +48101,10 @@
         <v>31</v>
       </c>
       <c r="F2335" s="7" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="2336" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="2336" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2336">
         <v>41093949</v>
       </c>
@@ -48130,10 +48121,10 @@
         <v>31</v>
       </c>
       <c r="F2336" s="7" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="2337" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2337" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2337">
         <v>41093949</v>
       </c>
@@ -48150,7 +48141,7 @@
         <v>31</v>
       </c>
       <c r="F2337" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2338" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48230,10 +48221,10 @@
         <v>7</v>
       </c>
       <c r="F2341" s="7" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="2342" spans="1:6" x14ac:dyDescent="0.2">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="2342" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2342">
         <v>37017009</v>
       </c>
@@ -48290,7 +48281,7 @@
         <v>18</v>
       </c>
       <c r="F2344" s="7" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="2345" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48350,7 +48341,7 @@
         <v>22</v>
       </c>
       <c r="F2347" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2348" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48433,7 +48424,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2352" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2352" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2352">
         <v>41112839</v>
       </c>
@@ -48450,10 +48441,10 @@
         <v>31</v>
       </c>
       <c r="F2352" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2353" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2353" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2353">
         <v>41112839</v>
       </c>
@@ -48470,7 +48461,7 @@
         <v>31</v>
       </c>
       <c r="F2353" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2354" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48533,7 +48524,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2357" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2357" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2357">
         <v>41129268</v>
       </c>
@@ -48550,10 +48541,10 @@
         <v>7</v>
       </c>
       <c r="F2357" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2358" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2358" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2358">
         <v>37938856</v>
       </c>
@@ -48570,7 +48561,7 @@
         <v>7</v>
       </c>
       <c r="F2358" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2359" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48590,7 +48581,7 @@
         <v>18</v>
       </c>
       <c r="F2359" s="7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2360" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48670,7 +48661,7 @@
         <v>22</v>
       </c>
       <c r="F2363" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2364" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48790,7 +48781,7 @@
         <v>31</v>
       </c>
       <c r="F2369" s="7" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="2370" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48853,7 +48844,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2373" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2373" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2373">
         <v>41130593</v>
       </c>
@@ -48870,10 +48861,10 @@
         <v>7</v>
       </c>
       <c r="F2373" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2374" spans="1:6" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2374" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2374">
         <v>37042390</v>
       </c>
@@ -48890,7 +48881,7 @@
         <v>7</v>
       </c>
       <c r="F2374" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2375" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48910,7 +48901,7 @@
         <v>18</v>
       </c>
       <c r="F2375" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2376" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48930,7 +48921,7 @@
         <v>18</v>
       </c>
       <c r="F2376" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2377" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48950,7 +48941,7 @@
         <v>22</v>
       </c>
       <c r="F2377" s="7" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="2378" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -48970,7 +48961,7 @@
         <v>22</v>
       </c>
       <c r="F2378" s="7" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2379" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -49030,7 +49021,7 @@
         <v>31</v>
       </c>
       <c r="F2381" s="7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2382" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -49090,7 +49081,7 @@
         <v>31</v>
       </c>
       <c r="F2384" s="7" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2385" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -49110,7 +49101,7 @@
         <v>31</v>
       </c>
       <c r="F2385" s="7" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2386" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -49193,7 +49184,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2390" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2390" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2390">
         <v>37515095</v>
       </c>
@@ -49250,7 +49241,7 @@
         <v>18</v>
       </c>
       <c r="F2392" s="7" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2393" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -49270,7 +49261,7 @@
         <v>22</v>
       </c>
       <c r="F2393" s="7" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="2394" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -49310,7 +49301,7 @@
         <v>22</v>
       </c>
       <c r="F2395" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2396" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -49330,7 +49321,7 @@
         <v>22</v>
       </c>
       <c r="F2396" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2397" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -49413,7 +49404,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2401" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2401" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2401">
         <v>41140464</v>
       </c>
@@ -49430,19 +49421,16 @@
         <v>31</v>
       </c>
       <c r="F2401" s="7" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F2401" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
+    <filterColumn colId="5">
       <filters>
-        <filter val="5"/>
+        <filter val="None"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:F2390">
-      <sortCondition ref="F1:F2401"/>
-    </sortState>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F1921">
     <sortCondition ref="A2:A1921"/>

</xml_diff>

<commit_message>
update ground truth and merged answers
</commit_message>
<xml_diff>
--- a/advanced-prompting/csv/ground_truth.xlsx
+++ b/advanced-prompting/csv/ground_truth.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kaimingtao/HIVDB/chat_HIVDB_paper/advanced-prompting/csv/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{541414FF-EA9A-1A44-9E62-A25288B9826B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96212146-5994-1D4D-9663-D08BDAAB3D8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4240" yWindow="600" windowWidth="37460" windowHeight="20800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15260" yWindow="500" windowWidth="37460" windowHeight="20800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9468" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9469" uniqueCount="312">
   <si>
     <t>PMID</t>
   </si>
@@ -231,9 +231,6 @@
   </si>
   <si>
     <t>NNRTI, INSTI</t>
-  </si>
-  <si>
-    <t>US</t>
   </si>
   <si>
     <t>2021-2022</t>
@@ -686,9 +683,6 @@
     <t>3TC, TDF, EFV, LPV/r, EVG, ABC, DTG</t>
   </si>
   <si>
-    <t>South America, Africa, USA, Asia, Australia, Europe</t>
-  </si>
-  <si>
     <t>EFV, DTG, TDF, 3TC</t>
   </si>
   <si>
@@ -972,6 +966,12 @@
   </si>
   <si>
     <t xml:space="preserve"> None</t>
+  </si>
+  <si>
+    <t>Not Reported</t>
+  </si>
+  <si>
+    <t>South America, Africa, USA</t>
   </si>
 </sst>
 </file>
@@ -1443,7 +1443,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -1963,7 +1963,7 @@
         <v>22</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -4183,7 +4183,7 @@
         <v>22</v>
       </c>
       <c r="F138" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.2">
@@ -5062,8 +5062,8 @@
       <c r="E182" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F182" s="9">
-        <v>1</v>
+      <c r="F182" s="9" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.2">
@@ -6963,7 +6963,7 @@
         <v>7</v>
       </c>
       <c r="F277" s="9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="278" spans="1:6" x14ac:dyDescent="0.2">
@@ -7843,7 +7843,7 @@
         <v>31</v>
       </c>
       <c r="F321" s="9" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="322" spans="1:6" x14ac:dyDescent="0.2">
@@ -7963,7 +7963,7 @@
         <v>18</v>
       </c>
       <c r="F327" s="9" t="s">
-        <v>65</v>
+        <v>310</v>
       </c>
     </row>
     <row r="328" spans="1:6" x14ac:dyDescent="0.2">
@@ -7983,7 +7983,7 @@
         <v>18</v>
       </c>
       <c r="F328" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="329" spans="1:6" x14ac:dyDescent="0.2">
@@ -8283,7 +8283,7 @@
         <v>18</v>
       </c>
       <c r="F343" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="344" spans="1:6" x14ac:dyDescent="0.2">
@@ -8303,7 +8303,7 @@
         <v>18</v>
       </c>
       <c r="F344" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="345" spans="1:6" x14ac:dyDescent="0.2">
@@ -8463,7 +8463,7 @@
         <v>31</v>
       </c>
       <c r="F352" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="353" spans="1:6" x14ac:dyDescent="0.2">
@@ -8483,7 +8483,7 @@
         <v>31</v>
       </c>
       <c r="F353" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="354" spans="1:6" x14ac:dyDescent="0.2">
@@ -8883,7 +8883,7 @@
         <v>7</v>
       </c>
       <c r="F373" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="374" spans="1:6" x14ac:dyDescent="0.2">
@@ -8923,7 +8923,7 @@
         <v>18</v>
       </c>
       <c r="F375" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="376" spans="1:6" x14ac:dyDescent="0.2">
@@ -8943,7 +8943,7 @@
         <v>18</v>
       </c>
       <c r="F376" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="377" spans="1:6" x14ac:dyDescent="0.2">
@@ -9123,7 +9123,7 @@
         <v>31</v>
       </c>
       <c r="F385" s="9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="386" spans="1:6" x14ac:dyDescent="0.2">
@@ -9563,7 +9563,7 @@
         <v>18</v>
       </c>
       <c r="F407" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="408" spans="1:6" x14ac:dyDescent="0.2">
@@ -9583,7 +9583,7 @@
         <v>18</v>
       </c>
       <c r="F408" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="409" spans="1:6" x14ac:dyDescent="0.2">
@@ -9883,7 +9883,7 @@
         <v>18</v>
       </c>
       <c r="F423" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="424" spans="1:6" x14ac:dyDescent="0.2">
@@ -10063,7 +10063,7 @@
         <v>31</v>
       </c>
       <c r="F432" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="433" spans="1:6" x14ac:dyDescent="0.2">
@@ -10083,7 +10083,7 @@
         <v>31</v>
       </c>
       <c r="F433" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="434" spans="1:6" x14ac:dyDescent="0.2">
@@ -10183,7 +10183,7 @@
         <v>7</v>
       </c>
       <c r="F438" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="439" spans="1:6" x14ac:dyDescent="0.2">
@@ -10203,7 +10203,7 @@
         <v>18</v>
       </c>
       <c r="F439" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="440" spans="1:6" x14ac:dyDescent="0.2">
@@ -10403,7 +10403,7 @@
         <v>31</v>
       </c>
       <c r="F449" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="450" spans="1:6" x14ac:dyDescent="0.2">
@@ -10523,7 +10523,7 @@
         <v>18</v>
       </c>
       <c r="F455" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="456" spans="1:6" x14ac:dyDescent="0.2">
@@ -10543,7 +10543,7 @@
         <v>18</v>
       </c>
       <c r="F456" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="457" spans="1:6" x14ac:dyDescent="0.2">
@@ -10723,7 +10723,7 @@
         <v>31</v>
       </c>
       <c r="F465" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="466" spans="1:6" x14ac:dyDescent="0.2">
@@ -10823,7 +10823,7 @@
         <v>7</v>
       </c>
       <c r="F470" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="471" spans="1:6" x14ac:dyDescent="0.2">
@@ -11043,7 +11043,7 @@
         <v>31</v>
       </c>
       <c r="F481" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="482" spans="1:6" x14ac:dyDescent="0.2">
@@ -11183,7 +11183,7 @@
         <v>18</v>
       </c>
       <c r="F488" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="489" spans="1:6" x14ac:dyDescent="0.2">
@@ -11263,7 +11263,7 @@
         <v>22</v>
       </c>
       <c r="F492" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="493" spans="1:6" x14ac:dyDescent="0.2">
@@ -11343,7 +11343,7 @@
         <v>31</v>
       </c>
       <c r="F496" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="497" spans="1:6" x14ac:dyDescent="0.2">
@@ -11363,7 +11363,7 @@
         <v>31</v>
       </c>
       <c r="F497" s="9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="498" spans="1:6" x14ac:dyDescent="0.2">
@@ -11463,7 +11463,7 @@
         <v>7</v>
       </c>
       <c r="F502" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="503" spans="1:6" x14ac:dyDescent="0.2">
@@ -11483,7 +11483,7 @@
         <v>18</v>
       </c>
       <c r="F503" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="504" spans="1:6" x14ac:dyDescent="0.2">
@@ -11503,7 +11503,7 @@
         <v>18</v>
       </c>
       <c r="F504" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="505" spans="1:6" x14ac:dyDescent="0.2">
@@ -11683,7 +11683,7 @@
         <v>31</v>
       </c>
       <c r="F513" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="514" spans="1:6" x14ac:dyDescent="0.2">
@@ -11803,7 +11803,7 @@
         <v>18</v>
       </c>
       <c r="F519" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="520" spans="1:6" x14ac:dyDescent="0.2">
@@ -12143,7 +12143,7 @@
         <v>18</v>
       </c>
       <c r="F536" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="537" spans="1:6" x14ac:dyDescent="0.2">
@@ -12443,7 +12443,7 @@
         <v>18</v>
       </c>
       <c r="F551" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="552" spans="1:6" x14ac:dyDescent="0.2">
@@ -12643,7 +12643,7 @@
         <v>31</v>
       </c>
       <c r="F561" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="562" spans="1:6" x14ac:dyDescent="0.2">
@@ -13083,7 +13083,7 @@
         <v>18</v>
       </c>
       <c r="F583" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="584" spans="1:6" x14ac:dyDescent="0.2">
@@ -13103,7 +13103,7 @@
         <v>18</v>
       </c>
       <c r="F584" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="585" spans="1:6" x14ac:dyDescent="0.2">
@@ -13363,7 +13363,7 @@
         <v>7</v>
       </c>
       <c r="F597" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="598" spans="1:6" x14ac:dyDescent="0.2">
@@ -13403,7 +13403,7 @@
         <v>18</v>
       </c>
       <c r="F599" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="600" spans="1:6" x14ac:dyDescent="0.2">
@@ -13423,7 +13423,7 @@
         <v>18</v>
       </c>
       <c r="F600" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="601" spans="1:6" x14ac:dyDescent="0.2">
@@ -13503,7 +13503,7 @@
         <v>22</v>
       </c>
       <c r="F604" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="605" spans="1:6" x14ac:dyDescent="0.2">
@@ -13583,7 +13583,7 @@
         <v>31</v>
       </c>
       <c r="F608" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="609" spans="1:6" x14ac:dyDescent="0.2">
@@ -13783,7 +13783,7 @@
         <v>22</v>
       </c>
       <c r="F618" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="619" spans="1:6" x14ac:dyDescent="0.2">
@@ -13803,7 +13803,7 @@
         <v>22</v>
       </c>
       <c r="F619" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="620" spans="1:6" x14ac:dyDescent="0.2">
@@ -14143,7 +14143,7 @@
         <v>22</v>
       </c>
       <c r="F636" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="637" spans="1:6" x14ac:dyDescent="0.2">
@@ -14243,7 +14243,7 @@
         <v>31</v>
       </c>
       <c r="F641" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="642" spans="1:6" x14ac:dyDescent="0.2">
@@ -14363,7 +14363,7 @@
         <v>18</v>
       </c>
       <c r="F647" s="9" t="s">
-        <v>51</v>
+        <v>14</v>
       </c>
     </row>
     <row r="648" spans="1:6" x14ac:dyDescent="0.2">
@@ -14383,7 +14383,7 @@
         <v>18</v>
       </c>
       <c r="F648" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="649" spans="1:6" x14ac:dyDescent="0.2">
@@ -14443,7 +14443,7 @@
         <v>22</v>
       </c>
       <c r="F651" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="652" spans="1:6" x14ac:dyDescent="0.2">
@@ -14743,7 +14743,7 @@
         <v>22</v>
       </c>
       <c r="F666" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="667" spans="1:6" x14ac:dyDescent="0.2">
@@ -15303,7 +15303,7 @@
         <v>7</v>
       </c>
       <c r="F694" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="695" spans="1:6" x14ac:dyDescent="0.2">
@@ -15323,7 +15323,7 @@
         <v>18</v>
       </c>
       <c r="F695" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="696" spans="1:6" x14ac:dyDescent="0.2">
@@ -15343,7 +15343,7 @@
         <v>18</v>
       </c>
       <c r="F696" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="697" spans="1:6" x14ac:dyDescent="0.2">
@@ -15403,7 +15403,7 @@
         <v>22</v>
       </c>
       <c r="F699" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="700" spans="1:6" x14ac:dyDescent="0.2">
@@ -15523,7 +15523,7 @@
         <v>31</v>
       </c>
       <c r="F705" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="706" spans="1:6" x14ac:dyDescent="0.2">
@@ -15643,7 +15643,7 @@
         <v>18</v>
       </c>
       <c r="F711" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="712" spans="1:6" x14ac:dyDescent="0.2">
@@ -15663,7 +15663,7 @@
         <v>18</v>
       </c>
       <c r="F712" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="713" spans="1:6" x14ac:dyDescent="0.2">
@@ -15963,7 +15963,7 @@
         <v>18</v>
       </c>
       <c r="F727" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="728" spans="1:6" x14ac:dyDescent="0.2">
@@ -15983,7 +15983,7 @@
         <v>18</v>
       </c>
       <c r="F728" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="729" spans="1:6" x14ac:dyDescent="0.2">
@@ -16023,7 +16023,7 @@
         <v>22</v>
       </c>
       <c r="F730" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="731" spans="1:6" x14ac:dyDescent="0.2">
@@ -16043,7 +16043,7 @@
         <v>22</v>
       </c>
       <c r="F731" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="732" spans="1:6" x14ac:dyDescent="0.2">
@@ -16163,7 +16163,7 @@
         <v>31</v>
       </c>
       <c r="F737" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="738" spans="1:6" x14ac:dyDescent="0.2">
@@ -16263,7 +16263,7 @@
         <v>7</v>
       </c>
       <c r="F742" s="9" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="743" spans="1:6" x14ac:dyDescent="0.2">
@@ -16283,7 +16283,7 @@
         <v>18</v>
       </c>
       <c r="F743" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="744" spans="1:6" x14ac:dyDescent="0.2">
@@ -16303,7 +16303,7 @@
         <v>18</v>
       </c>
       <c r="F744" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="745" spans="1:6" x14ac:dyDescent="0.2">
@@ -16483,7 +16483,7 @@
         <v>31</v>
       </c>
       <c r="F753" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="754" spans="1:6" x14ac:dyDescent="0.2">
@@ -17203,7 +17203,7 @@
         <v>7</v>
       </c>
       <c r="F789" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="790" spans="1:6" x14ac:dyDescent="0.2">
@@ -17543,7 +17543,7 @@
         <v>7</v>
       </c>
       <c r="F806" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="807" spans="1:6" x14ac:dyDescent="0.2">
@@ -17563,7 +17563,7 @@
         <v>18</v>
       </c>
       <c r="F807" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="808" spans="1:6" x14ac:dyDescent="0.2">
@@ -17583,7 +17583,7 @@
         <v>18</v>
       </c>
       <c r="F808" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="809" spans="1:6" x14ac:dyDescent="0.2">
@@ -17643,7 +17643,7 @@
         <v>22</v>
       </c>
       <c r="F811" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="812" spans="1:6" x14ac:dyDescent="0.2">
@@ -17663,7 +17663,7 @@
         <v>22</v>
       </c>
       <c r="F812" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="813" spans="1:6" x14ac:dyDescent="0.2">
@@ -17763,7 +17763,7 @@
         <v>31</v>
       </c>
       <c r="F817" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="818" spans="1:6" x14ac:dyDescent="0.2">
@@ -17883,7 +17883,7 @@
         <v>18</v>
       </c>
       <c r="F823" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="824" spans="1:6" x14ac:dyDescent="0.2">
@@ -17903,7 +17903,7 @@
         <v>18</v>
       </c>
       <c r="F824" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="825" spans="1:6" x14ac:dyDescent="0.2">
@@ -18203,7 +18203,7 @@
         <v>18</v>
       </c>
       <c r="F839" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="840" spans="1:6" x14ac:dyDescent="0.2">
@@ -18283,7 +18283,7 @@
         <v>22</v>
       </c>
       <c r="F843" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="844" spans="1:6" x14ac:dyDescent="0.2">
@@ -18523,7 +18523,7 @@
         <v>18</v>
       </c>
       <c r="F855" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="856" spans="1:6" x14ac:dyDescent="0.2">
@@ -18543,7 +18543,7 @@
         <v>18</v>
       </c>
       <c r="F856" s="9" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="857" spans="1:6" x14ac:dyDescent="0.2">
@@ -18803,7 +18803,7 @@
         <v>7</v>
       </c>
       <c r="F869" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="870" spans="1:6" x14ac:dyDescent="0.2">
@@ -18863,7 +18863,7 @@
         <v>18</v>
       </c>
       <c r="F872" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="873" spans="1:6" x14ac:dyDescent="0.2">
@@ -18903,7 +18903,7 @@
         <v>22</v>
       </c>
       <c r="F874" s="9" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="875" spans="1:6" x14ac:dyDescent="0.2">
@@ -19123,7 +19123,7 @@
         <v>7</v>
       </c>
       <c r="F885" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="886" spans="1:6" x14ac:dyDescent="0.2">
@@ -19143,7 +19143,7 @@
         <v>7</v>
       </c>
       <c r="F886" s="9" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="887" spans="1:6" x14ac:dyDescent="0.2">
@@ -19163,7 +19163,7 @@
         <v>18</v>
       </c>
       <c r="F887" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="888" spans="1:6" x14ac:dyDescent="0.2">
@@ -19183,7 +19183,7 @@
         <v>18</v>
       </c>
       <c r="F888" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="889" spans="1:6" x14ac:dyDescent="0.2">
@@ -19223,7 +19223,7 @@
         <v>22</v>
       </c>
       <c r="F890" s="9" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="891" spans="1:6" x14ac:dyDescent="0.2">
@@ -19683,7 +19683,7 @@
         <v>31</v>
       </c>
       <c r="F913" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="914" spans="1:6" x14ac:dyDescent="0.2">
@@ -20203,7 +20203,7 @@
         <v>22</v>
       </c>
       <c r="F939" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="940" spans="1:6" x14ac:dyDescent="0.2">
@@ -20223,7 +20223,7 @@
         <v>22</v>
       </c>
       <c r="F940" s="9" t="s">
-        <v>307</v>
+        <v>44</v>
       </c>
     </row>
     <row r="941" spans="1:6" x14ac:dyDescent="0.2">
@@ -20323,7 +20323,7 @@
         <v>31</v>
       </c>
       <c r="F945" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="946" spans="1:6" x14ac:dyDescent="0.2">
@@ -20463,7 +20463,7 @@
         <v>18</v>
       </c>
       <c r="F952" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="953" spans="1:6" x14ac:dyDescent="0.2">
@@ -20523,7 +20523,7 @@
         <v>22</v>
       </c>
       <c r="F955" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="956" spans="1:6" x14ac:dyDescent="0.2">
@@ -20763,7 +20763,7 @@
         <v>18</v>
       </c>
       <c r="F967" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="968" spans="1:6" x14ac:dyDescent="0.2">
@@ -20783,7 +20783,7 @@
         <v>18</v>
       </c>
       <c r="F968" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="969" spans="1:6" x14ac:dyDescent="0.2">
@@ -21083,7 +21083,7 @@
         <v>18</v>
       </c>
       <c r="F983" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="984" spans="1:6" x14ac:dyDescent="0.2">
@@ -21103,7 +21103,7 @@
         <v>18</v>
       </c>
       <c r="F984" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="985" spans="1:6" x14ac:dyDescent="0.2">
@@ -21283,7 +21283,7 @@
         <v>31</v>
       </c>
       <c r="F993" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="994" spans="1:6" x14ac:dyDescent="0.2">
@@ -21383,7 +21383,7 @@
         <v>7</v>
       </c>
       <c r="F998" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="999" spans="1:6" x14ac:dyDescent="0.2">
@@ -21403,7 +21403,7 @@
         <v>18</v>
       </c>
       <c r="F999" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="1000" spans="1:6" x14ac:dyDescent="0.2">
@@ -21463,7 +21463,7 @@
         <v>22</v>
       </c>
       <c r="F1002" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="1003" spans="1:6" x14ac:dyDescent="0.2">
@@ -21483,7 +21483,7 @@
         <v>22</v>
       </c>
       <c r="F1003" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="1004" spans="1:6" x14ac:dyDescent="0.2">
@@ -21603,7 +21603,7 @@
         <v>31</v>
       </c>
       <c r="F1009" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="1010" spans="1:6" x14ac:dyDescent="0.2">
@@ -21703,7 +21703,7 @@
         <v>7</v>
       </c>
       <c r="F1014" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="1015" spans="1:6" x14ac:dyDescent="0.2">
@@ -21723,7 +21723,7 @@
         <v>18</v>
       </c>
       <c r="F1015" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="1016" spans="1:6" x14ac:dyDescent="0.2">
@@ -21743,7 +21743,7 @@
         <v>18</v>
       </c>
       <c r="F1016" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="1017" spans="1:6" x14ac:dyDescent="0.2">
@@ -21923,7 +21923,7 @@
         <v>31</v>
       </c>
       <c r="F1025" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="1026" spans="1:6" x14ac:dyDescent="0.2">
@@ -22003,7 +22003,7 @@
         <v>7</v>
       </c>
       <c r="F1029" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="1030" spans="1:6" x14ac:dyDescent="0.2">
@@ -22043,7 +22043,7 @@
         <v>18</v>
       </c>
       <c r="F1031" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="1032" spans="1:6" x14ac:dyDescent="0.2">
@@ -22063,7 +22063,7 @@
         <v>18</v>
       </c>
       <c r="F1032" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="1033" spans="1:6" x14ac:dyDescent="0.2">
@@ -22323,7 +22323,7 @@
         <v>7</v>
       </c>
       <c r="F1045" s="9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="1046" spans="1:6" x14ac:dyDescent="0.2">
@@ -22343,7 +22343,7 @@
         <v>7</v>
       </c>
       <c r="F1046" s="9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="1047" spans="1:6" x14ac:dyDescent="0.2">
@@ -22363,7 +22363,7 @@
         <v>18</v>
       </c>
       <c r="F1047" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="1048" spans="1:6" x14ac:dyDescent="0.2">
@@ -22383,7 +22383,7 @@
         <v>18</v>
       </c>
       <c r="F1048" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="1049" spans="1:6" x14ac:dyDescent="0.2">
@@ -22563,7 +22563,7 @@
         <v>31</v>
       </c>
       <c r="F1057" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="1058" spans="1:6" x14ac:dyDescent="0.2">
@@ -22683,7 +22683,7 @@
         <v>18</v>
       </c>
       <c r="F1063" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="1064" spans="1:6" x14ac:dyDescent="0.2">
@@ -22703,7 +22703,7 @@
         <v>18</v>
       </c>
       <c r="F1064" s="9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="1065" spans="1:6" x14ac:dyDescent="0.2">
@@ -22763,7 +22763,7 @@
         <v>22</v>
       </c>
       <c r="F1067" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="1068" spans="1:6" x14ac:dyDescent="0.2">
@@ -23323,7 +23323,7 @@
         <v>18</v>
       </c>
       <c r="F1095" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="1096" spans="1:6" x14ac:dyDescent="0.2">
@@ -23343,7 +23343,7 @@
         <v>18</v>
       </c>
       <c r="F1096" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="1097" spans="1:6" x14ac:dyDescent="0.2">
@@ -23503,7 +23503,7 @@
         <v>31</v>
       </c>
       <c r="F1104" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="1105" spans="1:6" x14ac:dyDescent="0.2">
@@ -23523,7 +23523,7 @@
         <v>31</v>
       </c>
       <c r="F1105" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="1106" spans="1:6" x14ac:dyDescent="0.2">
@@ -23603,7 +23603,7 @@
         <v>7</v>
       </c>
       <c r="F1109" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="1110" spans="1:6" x14ac:dyDescent="0.2">
@@ -23663,7 +23663,7 @@
         <v>18</v>
       </c>
       <c r="F1112" s="9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="1113" spans="1:6" x14ac:dyDescent="0.2">
@@ -24283,7 +24283,7 @@
         <v>18</v>
       </c>
       <c r="F1143" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="1144" spans="1:6" x14ac:dyDescent="0.2">
@@ -24303,7 +24303,7 @@
         <v>18</v>
       </c>
       <c r="F1144" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="1145" spans="1:6" x14ac:dyDescent="0.2">
@@ -24583,7 +24583,7 @@
         <v>7</v>
       </c>
       <c r="F1158" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="1159" spans="1:6" x14ac:dyDescent="0.2">
@@ -24603,7 +24603,7 @@
         <v>18</v>
       </c>
       <c r="F1159" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="1160" spans="1:6" x14ac:dyDescent="0.2">
@@ -24623,7 +24623,7 @@
         <v>18</v>
       </c>
       <c r="F1160" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="1161" spans="1:6" x14ac:dyDescent="0.2">
@@ -24803,7 +24803,7 @@
         <v>31</v>
       </c>
       <c r="F1169" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="1170" spans="1:6" x14ac:dyDescent="0.2">
@@ -24923,7 +24923,7 @@
         <v>18</v>
       </c>
       <c r="F1175" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="1176" spans="1:6" x14ac:dyDescent="0.2">
@@ -24943,7 +24943,7 @@
         <v>18</v>
       </c>
       <c r="F1176" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="1177" spans="1:6" x14ac:dyDescent="0.2">
@@ -24983,7 +24983,7 @@
         <v>22</v>
       </c>
       <c r="F1178" s="9" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="1179" spans="1:6" x14ac:dyDescent="0.2">
@@ -25003,7 +25003,7 @@
         <v>22</v>
       </c>
       <c r="F1179" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="1180" spans="1:6" x14ac:dyDescent="0.2">
@@ -25123,7 +25123,7 @@
         <v>31</v>
       </c>
       <c r="F1185" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="1186" spans="1:6" x14ac:dyDescent="0.2">
@@ -25263,7 +25263,7 @@
         <v>18</v>
       </c>
       <c r="F1192" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="1193" spans="1:6" x14ac:dyDescent="0.2">
@@ -25583,7 +25583,7 @@
         <v>18</v>
       </c>
       <c r="F1208" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="1209" spans="1:6" x14ac:dyDescent="0.2">
@@ -25763,7 +25763,7 @@
         <v>31</v>
       </c>
       <c r="F1217" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="1218" spans="1:6" x14ac:dyDescent="0.2">
@@ -25843,7 +25843,7 @@
         <v>7</v>
       </c>
       <c r="F1221" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="1222" spans="1:6" x14ac:dyDescent="0.2">
@@ -25883,7 +25883,7 @@
         <v>18</v>
       </c>
       <c r="F1223" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="1224" spans="1:6" x14ac:dyDescent="0.2">
@@ -25903,7 +25903,7 @@
         <v>18</v>
       </c>
       <c r="F1224" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="1225" spans="1:6" x14ac:dyDescent="0.2">
@@ -26083,7 +26083,7 @@
         <v>31</v>
       </c>
       <c r="F1233" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="1234" spans="1:6" x14ac:dyDescent="0.2">
@@ -27143,7 +27143,7 @@
         <v>7</v>
       </c>
       <c r="F1286" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="1287" spans="1:6" x14ac:dyDescent="0.2">
@@ -27183,7 +27183,7 @@
         <v>18</v>
       </c>
       <c r="F1288" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="1289" spans="1:6" x14ac:dyDescent="0.2">
@@ -27463,7 +27463,7 @@
         <v>7</v>
       </c>
       <c r="F1302" s="9" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="1303" spans="1:6" x14ac:dyDescent="0.2">
@@ -27483,7 +27483,7 @@
         <v>18</v>
       </c>
       <c r="F1303" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="1304" spans="1:6" x14ac:dyDescent="0.2">
@@ -27503,7 +27503,7 @@
         <v>18</v>
       </c>
       <c r="F1304" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="1305" spans="1:6" x14ac:dyDescent="0.2">
@@ -27543,7 +27543,7 @@
         <v>22</v>
       </c>
       <c r="F1306" s="9" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="1307" spans="1:6" x14ac:dyDescent="0.2">
@@ -28123,7 +28123,7 @@
         <v>18</v>
       </c>
       <c r="F1335" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="1336" spans="1:6" x14ac:dyDescent="0.2">
@@ -28143,7 +28143,7 @@
         <v>18</v>
       </c>
       <c r="F1336" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="1337" spans="1:6" x14ac:dyDescent="0.2">
@@ -28223,7 +28223,7 @@
         <v>22</v>
       </c>
       <c r="F1340" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="1341" spans="1:6" x14ac:dyDescent="0.2">
@@ -28423,7 +28423,7 @@
         <v>7</v>
       </c>
       <c r="F1350" s="9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="1351" spans="1:6" x14ac:dyDescent="0.2">
@@ -28443,7 +28443,7 @@
         <v>18</v>
       </c>
       <c r="F1351" s="9" t="s">
-        <v>216</v>
+        <v>311</v>
       </c>
     </row>
     <row r="1352" spans="1:6" x14ac:dyDescent="0.2">
@@ -28463,7 +28463,7 @@
         <v>18</v>
       </c>
       <c r="F1352" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="1353" spans="1:6" x14ac:dyDescent="0.2">
@@ -28523,7 +28523,7 @@
         <v>22</v>
       </c>
       <c r="F1355" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="1356" spans="1:6" x14ac:dyDescent="0.2">
@@ -28743,7 +28743,7 @@
         <v>7</v>
       </c>
       <c r="F1366" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="1367" spans="1:6" x14ac:dyDescent="0.2">
@@ -28763,7 +28763,7 @@
         <v>18</v>
       </c>
       <c r="F1367" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="1368" spans="1:6" x14ac:dyDescent="0.2">
@@ -28783,7 +28783,7 @@
         <v>18</v>
       </c>
       <c r="F1368" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="1369" spans="1:6" x14ac:dyDescent="0.2">
@@ -28843,7 +28843,7 @@
         <v>22</v>
       </c>
       <c r="F1371" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="1372" spans="1:6" x14ac:dyDescent="0.2">
@@ -28863,7 +28863,7 @@
         <v>22</v>
       </c>
       <c r="F1372" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="1373" spans="1:6" x14ac:dyDescent="0.2">
@@ -29063,7 +29063,7 @@
         <v>7</v>
       </c>
       <c r="F1382" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="1383" spans="1:6" x14ac:dyDescent="0.2">
@@ -29083,7 +29083,7 @@
         <v>18</v>
       </c>
       <c r="F1383" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="1384" spans="1:6" x14ac:dyDescent="0.2">
@@ -29103,7 +29103,7 @@
         <v>18</v>
       </c>
       <c r="F1384" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="1385" spans="1:6" x14ac:dyDescent="0.2">
@@ -29143,7 +29143,7 @@
         <v>22</v>
       </c>
       <c r="F1386" s="9" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="1387" spans="1:6" x14ac:dyDescent="0.2">
@@ -29163,7 +29163,7 @@
         <v>22</v>
       </c>
       <c r="F1387" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="1388" spans="1:6" x14ac:dyDescent="0.2">
@@ -29283,7 +29283,7 @@
         <v>31</v>
       </c>
       <c r="F1393" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="1394" spans="1:6" x14ac:dyDescent="0.2">
@@ -29463,7 +29463,7 @@
         <v>22</v>
       </c>
       <c r="F1402" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="1403" spans="1:6" x14ac:dyDescent="0.2">
@@ -29723,7 +29723,7 @@
         <v>18</v>
       </c>
       <c r="F1415" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="1416" spans="1:6" x14ac:dyDescent="0.2">
@@ -29743,7 +29743,7 @@
         <v>18</v>
       </c>
       <c r="F1416" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="1417" spans="1:6" x14ac:dyDescent="0.2">
@@ -29923,7 +29923,7 @@
         <v>31</v>
       </c>
       <c r="F1425" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="1426" spans="1:6" x14ac:dyDescent="0.2">
@@ -30063,7 +30063,7 @@
         <v>18</v>
       </c>
       <c r="F1432" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="1433" spans="1:6" x14ac:dyDescent="0.2">
@@ -30323,7 +30323,7 @@
         <v>7</v>
       </c>
       <c r="F1445" s="9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="1446" spans="1:6" x14ac:dyDescent="0.2">
@@ -30363,7 +30363,7 @@
         <v>18</v>
       </c>
       <c r="F1447" s="9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="1448" spans="1:6" x14ac:dyDescent="0.2">
@@ -30663,7 +30663,7 @@
         <v>7</v>
       </c>
       <c r="F1462" s="9" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="1463" spans="1:6" x14ac:dyDescent="0.2">
@@ -30683,7 +30683,7 @@
         <v>18</v>
       </c>
       <c r="F1463" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="1464" spans="1:6" x14ac:dyDescent="0.2">
@@ -30703,7 +30703,7 @@
         <v>18</v>
       </c>
       <c r="F1464" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="1465" spans="1:6" x14ac:dyDescent="0.2">
@@ -30863,7 +30863,7 @@
         <v>31</v>
       </c>
       <c r="F1472" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="1473" spans="1:6" x14ac:dyDescent="0.2">
@@ -30883,7 +30883,7 @@
         <v>31</v>
       </c>
       <c r="F1473" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="1474" spans="1:6" x14ac:dyDescent="0.2">
@@ -31343,7 +31343,7 @@
         <v>18</v>
       </c>
       <c r="F1496" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="1497" spans="1:6" x14ac:dyDescent="0.2">
@@ -31403,7 +31403,7 @@
         <v>22</v>
       </c>
       <c r="F1499" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="1500" spans="1:6" x14ac:dyDescent="0.2">
@@ -31623,7 +31623,7 @@
         <v>7</v>
       </c>
       <c r="F1510" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="1511" spans="1:6" x14ac:dyDescent="0.2">
@@ -31663,7 +31663,7 @@
         <v>18</v>
       </c>
       <c r="F1512" s="9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="1513" spans="1:6" x14ac:dyDescent="0.2">
@@ -31943,7 +31943,7 @@
         <v>7</v>
       </c>
       <c r="F1526" s="9" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="1527" spans="1:6" x14ac:dyDescent="0.2">
@@ -31963,7 +31963,7 @@
         <v>18</v>
       </c>
       <c r="F1527" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="1528" spans="1:6" x14ac:dyDescent="0.2">
@@ -31983,7 +31983,7 @@
         <v>18</v>
       </c>
       <c r="F1528" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="1529" spans="1:6" x14ac:dyDescent="0.2">
@@ -32163,7 +32163,7 @@
         <v>31</v>
       </c>
       <c r="F1537" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="1538" spans="1:6" x14ac:dyDescent="0.2">
@@ -32263,7 +32263,7 @@
         <v>7</v>
       </c>
       <c r="F1542" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="1543" spans="1:6" x14ac:dyDescent="0.2">
@@ -32303,7 +32303,7 @@
         <v>18</v>
       </c>
       <c r="F1544" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="1545" spans="1:6" x14ac:dyDescent="0.2">
@@ -32483,7 +32483,7 @@
         <v>31</v>
       </c>
       <c r="F1553" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="1554" spans="1:6" x14ac:dyDescent="0.2">
@@ -32623,7 +32623,7 @@
         <v>18</v>
       </c>
       <c r="F1560" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="1561" spans="1:6" x14ac:dyDescent="0.2">
@@ -32983,7 +32983,7 @@
         <v>22</v>
       </c>
       <c r="F1578" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="1579" spans="1:6" x14ac:dyDescent="0.2">
@@ -33003,7 +33003,7 @@
         <v>22</v>
       </c>
       <c r="F1579" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="1580" spans="1:6" x14ac:dyDescent="0.2">
@@ -33123,7 +33123,7 @@
         <v>31</v>
       </c>
       <c r="F1585" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="1586" spans="1:6" x14ac:dyDescent="0.2">
@@ -33563,7 +33563,7 @@
         <v>18</v>
       </c>
       <c r="F1607" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="1608" spans="1:6" x14ac:dyDescent="0.2">
@@ -33583,7 +33583,7 @@
         <v>18</v>
       </c>
       <c r="F1608" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="1609" spans="1:6" x14ac:dyDescent="0.2">
@@ -34223,7 +34223,7 @@
         <v>18</v>
       </c>
       <c r="F1640" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="1641" spans="1:6" x14ac:dyDescent="0.2">
@@ -34403,7 +34403,7 @@
         <v>31</v>
       </c>
       <c r="F1649" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="1650" spans="1:6" x14ac:dyDescent="0.2">
@@ -34523,7 +34523,7 @@
         <v>18</v>
       </c>
       <c r="F1655" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="1656" spans="1:6" x14ac:dyDescent="0.2">
@@ -34723,7 +34723,7 @@
         <v>31</v>
       </c>
       <c r="F1665" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="1666" spans="1:6" x14ac:dyDescent="0.2">
@@ -35163,7 +35163,7 @@
         <v>18</v>
       </c>
       <c r="F1687" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="1688" spans="1:6" x14ac:dyDescent="0.2">
@@ -35183,7 +35183,7 @@
         <v>18</v>
       </c>
       <c r="F1688" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="1689" spans="1:6" x14ac:dyDescent="0.2">
@@ -35343,7 +35343,7 @@
         <v>31</v>
       </c>
       <c r="F1696" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="1697" spans="1:6" x14ac:dyDescent="0.2">
@@ -36443,7 +36443,7 @@
         <v>18</v>
       </c>
       <c r="F1751" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="1752" spans="1:6" x14ac:dyDescent="0.2">
@@ -36463,7 +36463,7 @@
         <v>18</v>
       </c>
       <c r="F1752" s="9" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="1753" spans="1:6" x14ac:dyDescent="0.2">
@@ -36503,7 +36503,7 @@
         <v>22</v>
       </c>
       <c r="F1754" s="9" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
     </row>
     <row r="1755" spans="1:6" x14ac:dyDescent="0.2">
@@ -36643,7 +36643,7 @@
         <v>31</v>
       </c>
       <c r="F1761" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="1762" spans="1:6" x14ac:dyDescent="0.2">
@@ -36863,7 +36863,7 @@
         <v>22</v>
       </c>
       <c r="F1772" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="1773" spans="1:6" x14ac:dyDescent="0.2">
@@ -36963,7 +36963,7 @@
         <v>31</v>
       </c>
       <c r="F1777" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="1778" spans="1:6" x14ac:dyDescent="0.2">
@@ -37083,7 +37083,7 @@
         <v>18</v>
       </c>
       <c r="F1783" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="1784" spans="1:6" x14ac:dyDescent="0.2">
@@ -37103,7 +37103,7 @@
         <v>18</v>
       </c>
       <c r="F1784" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="1785" spans="1:6" x14ac:dyDescent="0.2">
@@ -37283,7 +37283,7 @@
         <v>31</v>
       </c>
       <c r="F1793" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="1794" spans="1:6" x14ac:dyDescent="0.2">
@@ -37403,7 +37403,7 @@
         <v>18</v>
       </c>
       <c r="F1799" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="1800" spans="1:6" x14ac:dyDescent="0.2">
@@ -37423,7 +37423,7 @@
         <v>18</v>
       </c>
       <c r="F1800" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="1801" spans="1:6" x14ac:dyDescent="0.2">
@@ -37503,7 +37503,7 @@
         <v>22</v>
       </c>
       <c r="F1804" s="9" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="1805" spans="1:6" x14ac:dyDescent="0.2">
@@ -37683,7 +37683,7 @@
         <v>7</v>
       </c>
       <c r="F1813" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="1814" spans="1:6" x14ac:dyDescent="0.2">
@@ -37723,7 +37723,7 @@
         <v>18</v>
       </c>
       <c r="F1815" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="1816" spans="1:6" x14ac:dyDescent="0.2">
@@ -37743,7 +37743,7 @@
         <v>18</v>
       </c>
       <c r="F1816" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="1817" spans="1:6" x14ac:dyDescent="0.2">
@@ -37803,7 +37803,7 @@
         <v>22</v>
       </c>
       <c r="F1819" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="1820" spans="1:6" x14ac:dyDescent="0.2">
@@ -38883,7 +38883,7 @@
         <v>31</v>
       </c>
       <c r="F1873" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="1874" spans="1:6" x14ac:dyDescent="0.2">
@@ -39023,7 +39023,7 @@
         <v>18</v>
       </c>
       <c r="F1880" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="1881" spans="1:6" x14ac:dyDescent="0.2">
@@ -39103,7 +39103,7 @@
         <v>22</v>
       </c>
       <c r="F1884" s="9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="1885" spans="1:6" x14ac:dyDescent="0.2">
@@ -39383,7 +39383,7 @@
         <v>22</v>
       </c>
       <c r="F1898" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="1899" spans="1:6" x14ac:dyDescent="0.2">
@@ -39603,7 +39603,7 @@
         <v>7</v>
       </c>
       <c r="F1909" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="1910" spans="1:6" x14ac:dyDescent="0.2">
@@ -39703,7 +39703,7 @@
         <v>22</v>
       </c>
       <c r="F1914" s="9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="1915" spans="1:6" x14ac:dyDescent="0.2">
@@ -39923,7 +39923,7 @@
         <v>7</v>
       </c>
       <c r="F1925" s="5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1926" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -39963,7 +39963,7 @@
         <v>18</v>
       </c>
       <c r="F1927" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="1928" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -39983,7 +39983,7 @@
         <v>18</v>
       </c>
       <c r="F1928" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="1929" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40043,7 +40043,7 @@
         <v>22</v>
       </c>
       <c r="F1931" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="1932" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40163,7 +40163,7 @@
         <v>31</v>
       </c>
       <c r="F1937" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="1938" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40243,7 +40243,7 @@
         <v>7</v>
       </c>
       <c r="F1941" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="1942" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40283,7 +40283,7 @@
         <v>18</v>
       </c>
       <c r="F1943" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="1944" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40303,7 +40303,7 @@
         <v>18</v>
       </c>
       <c r="F1944" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="1945" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40343,7 +40343,7 @@
         <v>22</v>
       </c>
       <c r="F1946" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="1947" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -40363,7 +40363,7 @@
         <v>22</v>
       </c>
       <c r="F1947" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="1948" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40403,7 +40403,7 @@
         <v>31</v>
       </c>
       <c r="F1949" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="1950" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -40483,7 +40483,7 @@
         <v>31</v>
       </c>
       <c r="F1953" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="1954" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40563,7 +40563,7 @@
         <v>7</v>
       </c>
       <c r="F1957" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="1958" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40603,7 +40603,7 @@
         <v>18</v>
       </c>
       <c r="F1959" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="1960" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40623,7 +40623,7 @@
         <v>18</v>
       </c>
       <c r="F1960" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="1961" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40663,7 +40663,7 @@
         <v>22</v>
       </c>
       <c r="F1962" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="1963" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -40683,7 +40683,7 @@
         <v>22</v>
       </c>
       <c r="F1963" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="1964" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40803,7 +40803,7 @@
         <v>31</v>
       </c>
       <c r="F1969" s="5" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="1970" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40883,7 +40883,7 @@
         <v>7</v>
       </c>
       <c r="F1973" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="1974" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40923,7 +40923,7 @@
         <v>18</v>
       </c>
       <c r="F1975" s="5" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="1976" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40943,7 +40943,7 @@
         <v>18</v>
       </c>
       <c r="F1976" s="5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="1977" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40983,7 +40983,7 @@
         <v>22</v>
       </c>
       <c r="F1978" s="5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="1979" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -41003,7 +41003,7 @@
         <v>22</v>
       </c>
       <c r="F1979" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="1980" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41103,7 +41103,7 @@
         <v>31</v>
       </c>
       <c r="F1984" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="1985" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41123,7 +41123,7 @@
         <v>31</v>
       </c>
       <c r="F1985" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="1986" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41203,7 +41203,7 @@
         <v>7</v>
       </c>
       <c r="F1989" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="1990" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41243,7 +41243,7 @@
         <v>18</v>
       </c>
       <c r="F1991" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="1992" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41263,7 +41263,7 @@
         <v>18</v>
       </c>
       <c r="F1992" s="5" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="1993" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41303,7 +41303,7 @@
         <v>22</v>
       </c>
       <c r="F1994" s="5" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="1995" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -41323,7 +41323,7 @@
         <v>22</v>
       </c>
       <c r="F1995" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="1996" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41443,7 +41443,7 @@
         <v>31</v>
       </c>
       <c r="F2001" s="5" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2002" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41523,7 +41523,7 @@
         <v>7</v>
       </c>
       <c r="F2005" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2006" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41563,7 +41563,7 @@
         <v>18</v>
       </c>
       <c r="F2007" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2008" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41583,7 +41583,7 @@
         <v>18</v>
       </c>
       <c r="F2008" s="5" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2009" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41643,7 +41643,7 @@
         <v>22</v>
       </c>
       <c r="F2011" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2012" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41743,7 +41743,7 @@
         <v>31</v>
       </c>
       <c r="F2016" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2017" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41763,7 +41763,7 @@
         <v>31</v>
       </c>
       <c r="F2017" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2018" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41843,7 +41843,7 @@
         <v>7</v>
       </c>
       <c r="F2021" s="5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2022" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41883,7 +41883,7 @@
         <v>18</v>
       </c>
       <c r="F2023" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2024" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41903,7 +41903,7 @@
         <v>18</v>
       </c>
       <c r="F2024" s="5" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2025" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41943,7 +41943,7 @@
         <v>22</v>
       </c>
       <c r="F2026" s="5" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2027" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -41963,7 +41963,7 @@
         <v>22</v>
       </c>
       <c r="F2027" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2028" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42083,7 +42083,7 @@
         <v>31</v>
       </c>
       <c r="F2033" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2034" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42163,7 +42163,7 @@
         <v>7</v>
       </c>
       <c r="F2037" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2038" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42203,7 +42203,7 @@
         <v>18</v>
       </c>
       <c r="F2039" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="2040" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42223,7 +42223,7 @@
         <v>18</v>
       </c>
       <c r="F2040" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2041" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42403,7 +42403,7 @@
         <v>31</v>
       </c>
       <c r="F2049" s="5" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2050" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42483,7 +42483,7 @@
         <v>7</v>
       </c>
       <c r="F2053" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2054" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42523,7 +42523,7 @@
         <v>18</v>
       </c>
       <c r="F2055" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2056" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42543,7 +42543,7 @@
         <v>18</v>
       </c>
       <c r="F2056" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2057" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42603,7 +42603,7 @@
         <v>22</v>
       </c>
       <c r="F2059" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2060" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42723,7 +42723,7 @@
         <v>31</v>
       </c>
       <c r="F2065" s="5" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2066" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42803,7 +42803,7 @@
         <v>7</v>
       </c>
       <c r="F2069" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2070" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42843,7 +42843,7 @@
         <v>18</v>
       </c>
       <c r="F2071" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2072" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42863,7 +42863,7 @@
         <v>18</v>
       </c>
       <c r="F2072" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2073" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42903,7 +42903,7 @@
         <v>22</v>
       </c>
       <c r="F2074" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2075" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -42963,7 +42963,7 @@
         <v>31</v>
       </c>
       <c r="F2077" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="2078" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -43023,7 +43023,7 @@
         <v>31</v>
       </c>
       <c r="F2080" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2081" spans="1:6" ht="30" x14ac:dyDescent="0.2">
@@ -43043,7 +43043,7 @@
         <v>31</v>
       </c>
       <c r="F2081" s="5" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2082" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43123,7 +43123,7 @@
         <v>7</v>
       </c>
       <c r="F2085" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2086" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43163,7 +43163,7 @@
         <v>18</v>
       </c>
       <c r="F2087" s="5" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2088" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43183,7 +43183,7 @@
         <v>18</v>
       </c>
       <c r="F2088" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2089" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43223,7 +43223,7 @@
         <v>22</v>
       </c>
       <c r="F2090" s="5" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2091" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -43243,7 +43243,7 @@
         <v>22</v>
       </c>
       <c r="F2091" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2092" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43323,7 +43323,7 @@
         <v>31</v>
       </c>
       <c r="F2095" s="5" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2096" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -43363,7 +43363,7 @@
         <v>31</v>
       </c>
       <c r="F2097" s="5" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2098" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43443,7 +43443,7 @@
         <v>7</v>
       </c>
       <c r="F2101" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2102" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43463,7 +43463,7 @@
         <v>7</v>
       </c>
       <c r="F2102" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2103" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43483,7 +43483,7 @@
         <v>18</v>
       </c>
       <c r="F2103" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2104" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43503,7 +43503,7 @@
         <v>18</v>
       </c>
       <c r="F2104" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2105" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43543,7 +43543,7 @@
         <v>22</v>
       </c>
       <c r="F2106" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2107" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -43563,7 +43563,7 @@
         <v>22</v>
       </c>
       <c r="F2107" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2108" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43683,7 +43683,7 @@
         <v>31</v>
       </c>
       <c r="F2113" s="5" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2114" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43783,7 +43783,7 @@
         <v>7</v>
       </c>
       <c r="F2118" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2119" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43803,7 +43803,7 @@
         <v>18</v>
       </c>
       <c r="F2119" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2120" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43823,7 +43823,7 @@
         <v>18</v>
       </c>
       <c r="F2120" s="5" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2121" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43863,7 +43863,7 @@
         <v>22</v>
       </c>
       <c r="F2122" s="5" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2123" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -43883,7 +43883,7 @@
         <v>22</v>
       </c>
       <c r="F2123" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2124" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44003,7 +44003,7 @@
         <v>31</v>
       </c>
       <c r="F2129" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2130" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44083,7 +44083,7 @@
         <v>7</v>
       </c>
       <c r="F2133" s="5" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2134" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44143,7 +44143,7 @@
         <v>18</v>
       </c>
       <c r="F2136" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2137" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44183,7 +44183,7 @@
         <v>22</v>
       </c>
       <c r="F2138" s="5" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2139" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -44203,7 +44203,7 @@
         <v>22</v>
       </c>
       <c r="F2139" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2140" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44303,7 +44303,7 @@
         <v>31</v>
       </c>
       <c r="F2144" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2145" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44323,7 +44323,7 @@
         <v>31</v>
       </c>
       <c r="F2145" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2146" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44403,7 +44403,7 @@
         <v>7</v>
       </c>
       <c r="F2149" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2150" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44443,7 +44443,7 @@
         <v>18</v>
       </c>
       <c r="F2151" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2152" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44483,7 +44483,7 @@
         <v>22</v>
       </c>
       <c r="F2153" s="5" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2154" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44503,7 +44503,7 @@
         <v>22</v>
       </c>
       <c r="F2154" s="5" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2155" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -44523,7 +44523,7 @@
         <v>22</v>
       </c>
       <c r="F2155" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2156" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44543,7 +44543,7 @@
         <v>22</v>
       </c>
       <c r="F2156" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2157" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44623,7 +44623,7 @@
         <v>31</v>
       </c>
       <c r="F2160" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2161" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44643,7 +44643,7 @@
         <v>31</v>
       </c>
       <c r="F2161" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2162" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44723,7 +44723,7 @@
         <v>7</v>
       </c>
       <c r="F2165" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2166" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44763,7 +44763,7 @@
         <v>18</v>
       </c>
       <c r="F2167" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2168" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44823,7 +44823,7 @@
         <v>22</v>
       </c>
       <c r="F2170" s="5" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2171" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -44843,7 +44843,7 @@
         <v>22</v>
       </c>
       <c r="F2171" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2172" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44943,7 +44943,7 @@
         <v>31</v>
       </c>
       <c r="F2176" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2177" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44963,7 +44963,7 @@
         <v>31</v>
       </c>
       <c r="F2177" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2178" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45043,7 +45043,7 @@
         <v>7</v>
       </c>
       <c r="F2181" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2182" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45083,7 +45083,7 @@
         <v>18</v>
       </c>
       <c r="F2183" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2184" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45103,7 +45103,7 @@
         <v>18</v>
       </c>
       <c r="F2184" s="5" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="2185" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45143,7 +45143,7 @@
         <v>22</v>
       </c>
       <c r="F2186" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2187" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -45183,7 +45183,7 @@
         <v>22</v>
       </c>
       <c r="F2188" s="5" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2189" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45283,7 +45283,7 @@
         <v>31</v>
       </c>
       <c r="F2193" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2194" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45363,7 +45363,7 @@
         <v>7</v>
       </c>
       <c r="F2197" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2198" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45403,7 +45403,7 @@
         <v>18</v>
       </c>
       <c r="F2199" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2200" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45423,7 +45423,7 @@
         <v>18</v>
       </c>
       <c r="F2200" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2201" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45463,7 +45463,7 @@
         <v>22</v>
       </c>
       <c r="F2202" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2203" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -45583,7 +45583,7 @@
         <v>31</v>
       </c>
       <c r="F2208" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2209" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45603,7 +45603,7 @@
         <v>31</v>
       </c>
       <c r="F2209" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2210" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45623,7 +45623,7 @@
         <v>7</v>
       </c>
       <c r="F2210" s="5" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2211" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45683,7 +45683,7 @@
         <v>7</v>
       </c>
       <c r="F2213" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2214" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45703,7 +45703,7 @@
         <v>7</v>
       </c>
       <c r="F2214" s="5" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2215" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45723,7 +45723,7 @@
         <v>18</v>
       </c>
       <c r="F2215" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2216" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45743,7 +45743,7 @@
         <v>18</v>
       </c>
       <c r="F2216" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2217" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45783,7 +45783,7 @@
         <v>22</v>
       </c>
       <c r="F2218" s="5" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2219" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -45803,7 +45803,7 @@
         <v>22</v>
       </c>
       <c r="F2219" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2220" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45823,7 +45823,7 @@
         <v>22</v>
       </c>
       <c r="F2220" s="5" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2221" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45903,7 +45903,7 @@
         <v>31</v>
       </c>
       <c r="F2224" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2225" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45923,7 +45923,7 @@
         <v>31</v>
       </c>
       <c r="F2225" s="5" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2226" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46003,7 +46003,7 @@
         <v>7</v>
       </c>
       <c r="F2229" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2230" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46043,7 +46043,7 @@
         <v>18</v>
       </c>
       <c r="F2231" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2232" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46063,7 +46063,7 @@
         <v>18</v>
       </c>
       <c r="F2232" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2233" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46103,7 +46103,7 @@
         <v>22</v>
       </c>
       <c r="F2234" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2235" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -46123,7 +46123,7 @@
         <v>22</v>
       </c>
       <c r="F2235" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2236" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46223,7 +46223,7 @@
         <v>31</v>
       </c>
       <c r="F2240" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2241" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46243,7 +46243,7 @@
         <v>31</v>
       </c>
       <c r="F2241" s="5" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2242" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46303,7 +46303,7 @@
         <v>7</v>
       </c>
       <c r="F2244" s="5" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="2245" spans="1:6" ht="45" x14ac:dyDescent="0.2">
@@ -46323,7 +46323,7 @@
         <v>7</v>
       </c>
       <c r="F2245" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2246" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46363,7 +46363,7 @@
         <v>18</v>
       </c>
       <c r="F2247" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2248" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46383,7 +46383,7 @@
         <v>18</v>
       </c>
       <c r="F2248" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2249" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46423,7 +46423,7 @@
         <v>22</v>
       </c>
       <c r="F2250" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2251" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -46443,7 +46443,7 @@
         <v>22</v>
       </c>
       <c r="F2251" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2252" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46543,7 +46543,7 @@
         <v>31</v>
       </c>
       <c r="F2256" s="5" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2257" spans="1:6" ht="30" x14ac:dyDescent="0.2">
@@ -46563,7 +46563,7 @@
         <v>31</v>
       </c>
       <c r="F2257" s="5" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2258" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46643,7 +46643,7 @@
         <v>7</v>
       </c>
       <c r="F2261" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2262" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46683,7 +46683,7 @@
         <v>18</v>
       </c>
       <c r="F2263" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2264" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46703,7 +46703,7 @@
         <v>18</v>
       </c>
       <c r="F2264" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2265" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46743,7 +46743,7 @@
         <v>22</v>
       </c>
       <c r="F2266" s="5" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2267" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -46763,7 +46763,7 @@
         <v>22</v>
       </c>
       <c r="F2267" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2268" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46863,7 +46863,7 @@
         <v>31</v>
       </c>
       <c r="F2272" s="5" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2273" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46883,7 +46883,7 @@
         <v>31</v>
       </c>
       <c r="F2273" s="5" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="2274" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46963,7 +46963,7 @@
         <v>7</v>
       </c>
       <c r="F2277" s="6" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2278" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47003,7 +47003,7 @@
         <v>18</v>
       </c>
       <c r="F2279" s="6" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2280" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47023,7 +47023,7 @@
         <v>18</v>
       </c>
       <c r="F2280" s="6" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="2281" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47063,7 +47063,7 @@
         <v>22</v>
       </c>
       <c r="F2282" s="6" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2283" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -47083,7 +47083,7 @@
         <v>22</v>
       </c>
       <c r="F2283" s="6" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="2284" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47103,7 +47103,7 @@
         <v>22</v>
       </c>
       <c r="F2284" s="6" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="2285" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47183,7 +47183,7 @@
         <v>31</v>
       </c>
       <c r="F2288" s="6" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2289" spans="1:6" ht="30" x14ac:dyDescent="0.2">
@@ -47203,7 +47203,7 @@
         <v>31</v>
       </c>
       <c r="F2289" s="6" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2290" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47283,7 +47283,7 @@
         <v>7</v>
       </c>
       <c r="F2293" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2294" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47383,7 +47383,7 @@
         <v>22</v>
       </c>
       <c r="F2298" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2299" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -47403,7 +47403,7 @@
         <v>22</v>
       </c>
       <c r="F2299" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2300" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47483,7 +47483,7 @@
         <v>31</v>
       </c>
       <c r="F2303" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2304" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -47503,7 +47503,7 @@
         <v>31</v>
       </c>
       <c r="F2304" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2305" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47523,7 +47523,7 @@
         <v>31</v>
       </c>
       <c r="F2305" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2306" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47603,7 +47603,7 @@
         <v>7</v>
       </c>
       <c r="F2309" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2310" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47643,7 +47643,7 @@
         <v>18</v>
       </c>
       <c r="F2311" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2312" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47683,7 +47683,7 @@
         <v>22</v>
       </c>
       <c r="F2313" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="2314" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47703,7 +47703,7 @@
         <v>22</v>
       </c>
       <c r="F2314" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2315" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -47723,7 +47723,7 @@
         <v>22</v>
       </c>
       <c r="F2315" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2316" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47743,7 +47743,7 @@
         <v>22</v>
       </c>
       <c r="F2316" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2317" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47803,7 +47803,7 @@
         <v>31</v>
       </c>
       <c r="F2319" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2320" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -47823,7 +47823,7 @@
         <v>31</v>
       </c>
       <c r="F2320" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2321" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47843,7 +47843,7 @@
         <v>31</v>
       </c>
       <c r="F2321" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2322" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47863,7 +47863,7 @@
         <v>7</v>
       </c>
       <c r="F2322" s="5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="2323" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47903,7 +47903,7 @@
         <v>7</v>
       </c>
       <c r="F2324" s="5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="2325" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47923,7 +47923,7 @@
         <v>7</v>
       </c>
       <c r="F2325" s="5" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="2326" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47963,7 +47963,7 @@
         <v>18</v>
       </c>
       <c r="F2327" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2328" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47983,7 +47983,7 @@
         <v>18</v>
       </c>
       <c r="F2328" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2329" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48043,7 +48043,7 @@
         <v>22</v>
       </c>
       <c r="F2331" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2332" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48063,7 +48063,7 @@
         <v>22</v>
       </c>
       <c r="F2332" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2333" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48103,7 +48103,7 @@
         <v>31</v>
       </c>
       <c r="F2334" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2335" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -48123,7 +48123,7 @@
         <v>31</v>
       </c>
       <c r="F2335" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2336" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -48143,7 +48143,7 @@
         <v>31</v>
       </c>
       <c r="F2336" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2337" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48163,7 +48163,7 @@
         <v>31</v>
       </c>
       <c r="F2337" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2338" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48243,7 +48243,7 @@
         <v>7</v>
       </c>
       <c r="F2341" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2342" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48303,7 +48303,7 @@
         <v>18</v>
       </c>
       <c r="F2344" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="2345" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48363,7 +48363,7 @@
         <v>22</v>
       </c>
       <c r="F2347" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2348" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48463,7 +48463,7 @@
         <v>31</v>
       </c>
       <c r="F2352" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2353" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48483,7 +48483,7 @@
         <v>31</v>
       </c>
       <c r="F2353" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2354" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48563,7 +48563,7 @@
         <v>7</v>
       </c>
       <c r="F2357" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2358" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48603,7 +48603,7 @@
         <v>18</v>
       </c>
       <c r="F2359" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2360" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48663,7 +48663,7 @@
         <v>22</v>
       </c>
       <c r="F2362" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2363" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -48683,7 +48683,7 @@
         <v>22</v>
       </c>
       <c r="F2363" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2364" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48803,7 +48803,7 @@
         <v>31</v>
       </c>
       <c r="F2369" s="5" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2370" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48883,7 +48883,7 @@
         <v>7</v>
       </c>
       <c r="F2373" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2374" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48923,7 +48923,7 @@
         <v>18</v>
       </c>
       <c r="F2375" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2376" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48943,7 +48943,7 @@
         <v>18</v>
       </c>
       <c r="F2376" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2377" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48963,7 +48963,7 @@
         <v>22</v>
       </c>
       <c r="F2377" s="5" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2378" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48983,7 +48983,7 @@
         <v>22</v>
       </c>
       <c r="F2378" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="2379" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -49043,7 +49043,7 @@
         <v>31</v>
       </c>
       <c r="F2381" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2382" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -49103,7 +49103,7 @@
         <v>31</v>
       </c>
       <c r="F2384" s="5" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2385" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49123,7 +49123,7 @@
         <v>31</v>
       </c>
       <c r="F2385" s="5" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2386" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49223,7 +49223,7 @@
         <v>7</v>
       </c>
       <c r="F2390" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2391" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49243,7 +49243,7 @@
         <v>18</v>
       </c>
       <c r="F2391" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2392" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49263,7 +49263,7 @@
         <v>18</v>
       </c>
       <c r="F2392" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="2393" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49283,7 +49283,7 @@
         <v>22</v>
       </c>
       <c r="F2393" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2394" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49323,7 +49323,7 @@
         <v>22</v>
       </c>
       <c r="F2395" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2396" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49343,7 +49343,7 @@
         <v>22</v>
       </c>
       <c r="F2396" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2397" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49443,11 +49443,16 @@
         <v>31</v>
       </c>
       <c r="F2401" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F2401" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F2401" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F2401">
+      <sortCondition ref="A2:A2401"/>
+      <sortCondition ref="B2:B2401"/>
+    </sortState>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F1921">
     <sortCondition ref="A2:A1921"/>
     <sortCondition ref="B2:B1921"/>

</xml_diff>